<commit_message>
Add training results for B_bisrnet with WCE loss for folds 1 and 2
</commit_message>
<xml_diff>
--- a/results/SECOND_SCD_Results.xlsx
+++ b/results/SECOND_SCD_Results.xlsx
@@ -729,7 +729,7 @@
       <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="3476625"/>
+    <ext cx="8572500" cy="5172075"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -751,10 +751,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>41</row>
+      <row>50</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="3400425"/>
+    <ext cx="8572500" cy="5010150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -784,7 +784,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9334500" cy="4133850"/>
+    <ext cx="9334500" cy="6829425"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -806,10 +806,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>42</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9334500" cy="4133850"/>
+    <ext cx="9334500" cy="6829425"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -1368,8 +1368,8 @@
         </is>
       </c>
       <c r="B15" s="13" t="str">
-        <f>"15 of 36"</f>
-        <v>15 of 36</v>
+        <f>"36 of 36"</f>
+        <v>36 of 36</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
@@ -1462,13 +1462,13 @@
       </c>
       <c r="C45" s="14" t="n"/>
     </row>
-    <row r="46" ht="46.5" customHeight="1">
+    <row r="46" ht="60" customHeight="1">
       <c r="A46" s="15" t="n">
         <v>5</v>
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>Cross-validation (3 folds) confirms the order of the three designs in every fold. WCE + Dice, CE + Dice beat plain CE in all 3 folds. Highest mean so far: Bi-SRNet-lite + CE + Dice (14.38 ± 0.31). Techniques this close should be treated as ties.</t>
+          <t>Cross-validation (3 folds) confirms the order of the three designs in every fold. WCE + Dice, CE + Dice, Weighted CE, Median-freq, Class-balanced, WCE + Dice + rare sampling beat plain CE in all 3 folds. Highest mean so far: Bi-SRNet-lite + CE + Dice (14.38 ± 0.31). Techniques this close should be treated as ties.</t>
         </is>
       </c>
       <c r="C46" s="14" t="n"/>
@@ -4107,12 +4107,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Finish cross-validation; add 2 more seeds for the best configurations</t>
+          <t>Add 2 more seeds for the best configurations (cross-validation is done)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Every claim gets a mean ± std</t>
+          <t>Makes the small gaps between the top techniques testable</t>
         </is>
       </c>
       <c r="D6" s="58" t="inlineStr">
@@ -7471,7 +7471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M78"/>
+  <dimension ref="A1:M117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7499,14 +7499,14 @@
     <row r="2" ht="33" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What this sheet shows: each configuration is trained 3 times on different parts of the training data (1,582 train / 791 validation pairs each time) and scored on the same test split. Finished: 15 of 36 runs.</t>
+          <t>What this sheet shows: each configuration is trained 3 times on different parts of the training data (1,582 train / 791 validation pairs each time) and scored on the same test split. Finished: 36 of 36 runs.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="35.7" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Key takeaway: The order of the three designs holds in every fold. WCE + Dice, CE + Dice beat plain CE in all 3 folds. Highest mean so far: Bi-SRNet-lite + CE + Dice (14.38 ± 0.31). Techniques within about 0.3 SeK of each other are effectively tied.</t>
+          <t>Key takeaway: The order of the three designs holds in every fold. WCE + Dice, CE + Dice, Weighted CE, Median-freq, Class-balanced, WCE + Dice + rare sampling beat plain CE in all 3 folds. Highest mean so far: Bi-SRNet-lite + CE + Dice (14.38 ± 0.31). Techniques within about 0.3 SeK of each other are effectively tied.</t>
         </is>
       </c>
     </row>
@@ -7834,35 +7834,47 @@
           <t>Bi-SRNet-lite + Weighted CE</t>
         </is>
       </c>
-      <c r="B11" s="41" t="n"/>
-      <c r="C11" s="41" t="n"/>
-      <c r="D11" s="41" t="n"/>
+      <c r="B11" s="41" t="n">
+        <v>14.64664541715592</v>
+      </c>
+      <c r="C11" s="41" t="n">
+        <v>14.26148333562495</v>
+      </c>
+      <c r="D11" s="41" t="n">
+        <v>14.14211735890099</v>
+      </c>
       <c r="E11" s="44">
         <f>COUNT(B11:D11)</f>
-        <v>0.0</v>
-      </c>
-      <c r="F11" s="41" t="str">
+        <v>3.0</v>
+      </c>
+      <c r="F11" s="41">
         <f>IF(E11&gt;0,AVERAGE(B11:D11),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="G11" s="41" t="str">
+        <v>14.350082037227287</v>
+      </c>
+      <c r="G11" s="41">
         <f>IF(E11&gt;1,STDEV(B11:D11),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="H11" s="41" t="n"/>
-      <c r="I11" s="41" t="n"/>
-      <c r="J11" s="41" t="str">
+        <v>0.2636748714531543</v>
+      </c>
+      <c r="H11" s="41" t="n">
+        <v>14.88744218154656</v>
+      </c>
+      <c r="I11" s="41" t="n">
+        <v>22.94750718149162</v>
+      </c>
+      <c r="J11" s="41">
         <f>IF(AND(ISNUMBER(I11),ISNUMBER(H11)),I11-H11,"—")</f>
-        <v>—</v>
-      </c>
-      <c r="K11" s="33" t="n"/>
+        <v>8.06006499994506</v>
+      </c>
+      <c r="K11" s="33" t="n">
+        <v>0.009438503418193812</v>
+      </c>
       <c r="L11" s="54" t="str">
         <f>IF(AND(E11=3,E8=3),((B11&gt;B8)+(C11&gt;C8)+(D11&gt;D8))&amp;" of 3 folds","—")</f>
-        <v>—</v>
+        <v>3 of 3 folds</v>
       </c>
       <c r="M11" s="8" t="inlineStr">
         <is>
-          <t>not started yet</t>
+          <t>Mild overfitting</t>
         </is>
       </c>
     </row>
@@ -7872,35 +7884,47 @@
           <t>Bi-SRNet-lite + Median-freq</t>
         </is>
       </c>
-      <c r="B12" s="37" t="n"/>
-      <c r="C12" s="37" t="n"/>
-      <c r="D12" s="37" t="n"/>
+      <c r="B12" s="37" t="n">
+        <v>14.20669732292025</v>
+      </c>
+      <c r="C12" s="37" t="n">
+        <v>13.56942910926994</v>
+      </c>
+      <c r="D12" s="37" t="n">
+        <v>13.4191390301541</v>
+      </c>
       <c r="E12" s="40">
         <f>COUNT(B12:D12)</f>
-        <v>0.0</v>
-      </c>
-      <c r="F12" s="37" t="str">
+        <v>3.0</v>
+      </c>
+      <c r="F12" s="37">
         <f>IF(E12&gt;0,AVERAGE(B12:D12),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="G12" s="37" t="str">
+        <v>13.731755154114763</v>
+      </c>
+      <c r="G12" s="37">
         <f>IF(E12&gt;1,STDEV(B12:D12),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="H12" s="37" t="n"/>
-      <c r="I12" s="37" t="n"/>
-      <c r="J12" s="37" t="str">
+        <v>0.4181199884631282</v>
+      </c>
+      <c r="H12" s="37" t="n">
+        <v>14.3952469595525</v>
+      </c>
+      <c r="I12" s="37" t="n">
+        <v>20.99979076533944</v>
+      </c>
+      <c r="J12" s="37">
         <f>IF(AND(ISNUMBER(I12),ISNUMBER(H12)),I12-H12,"—")</f>
-        <v>—</v>
-      </c>
-      <c r="K12" s="31" t="n"/>
+        <v>6.604543805786941</v>
+      </c>
+      <c r="K12" s="31" t="n">
+        <v>0.01302308378053619</v>
+      </c>
       <c r="L12" s="50" t="str">
         <f>IF(AND(E12=3,E8=3),((B12&gt;B8)+(C12&gt;C8)+(D12&gt;D8))&amp;" of 3 folds","—")</f>
-        <v>—</v>
+        <v>3 of 3 folds</v>
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>not started yet</t>
+          <t>Mild overfitting</t>
         </is>
       </c>
     </row>
@@ -7910,35 +7934,47 @@
           <t>Bi-SRNet-lite + Class-balanced</t>
         </is>
       </c>
-      <c r="B13" s="41" t="n"/>
-      <c r="C13" s="41" t="n"/>
-      <c r="D13" s="41" t="n"/>
+      <c r="B13" s="41" t="n">
+        <v>14.37406026945466</v>
+      </c>
+      <c r="C13" s="41" t="n">
+        <v>14.38428715583249</v>
+      </c>
+      <c r="D13" s="41" t="n">
+        <v>13.68703818601729</v>
+      </c>
       <c r="E13" s="44">
         <f>COUNT(B13:D13)</f>
-        <v>0.0</v>
-      </c>
-      <c r="F13" s="41" t="str">
+        <v>3.0</v>
+      </c>
+      <c r="F13" s="41">
         <f>IF(E13&gt;0,AVERAGE(B13:D13),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="G13" s="41" t="str">
+        <v>14.148461870434813</v>
+      </c>
+      <c r="G13" s="41">
         <f>IF(E13&gt;1,STDEV(B13:D13),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="H13" s="41" t="n"/>
-      <c r="I13" s="41" t="n"/>
-      <c r="J13" s="41" t="str">
+        <v>0.39963734773833137</v>
+      </c>
+      <c r="H13" s="41" t="n">
+        <v>14.74727229161141</v>
+      </c>
+      <c r="I13" s="41" t="n">
+        <v>22.09379203256542</v>
+      </c>
+      <c r="J13" s="41">
         <f>IF(AND(ISNUMBER(I13),ISNUMBER(H13)),I13-H13,"—")</f>
-        <v>—</v>
-      </c>
-      <c r="K13" s="33" t="n"/>
+        <v>7.346519740954012</v>
+      </c>
+      <c r="K13" s="33" t="n">
+        <v>0.00931844022924809</v>
+      </c>
       <c r="L13" s="54" t="str">
         <f>IF(AND(E13=3,E8=3),((B13&gt;B8)+(C13&gt;C8)+(D13&gt;D8))&amp;" of 3 folds","—")</f>
-        <v>—</v>
+        <v>3 of 3 folds</v>
       </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
-          <t>not started yet</t>
+          <t>Mild overfitting</t>
         </is>
       </c>
     </row>
@@ -7948,35 +7984,47 @@
           <t>Bi-SRNet-lite + Focal</t>
         </is>
       </c>
-      <c r="B14" s="37" t="n"/>
-      <c r="C14" s="37" t="n"/>
-      <c r="D14" s="37" t="n"/>
+      <c r="B14" s="37" t="n">
+        <v>13.34032062207497</v>
+      </c>
+      <c r="C14" s="37" t="n">
+        <v>13.43639077930197</v>
+      </c>
+      <c r="D14" s="37" t="n">
+        <v>13.27131493006328</v>
+      </c>
       <c r="E14" s="40">
         <f>COUNT(B14:D14)</f>
-        <v>0.0</v>
-      </c>
-      <c r="F14" s="37" t="str">
+        <v>3.0</v>
+      </c>
+      <c r="F14" s="37">
         <f>IF(E14&gt;0,AVERAGE(B14:D14),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="G14" s="37" t="str">
+        <v>13.349342110480073</v>
+      </c>
+      <c r="G14" s="37">
         <f>IF(E14&gt;1,STDEV(B14:D14),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="H14" s="37" t="n"/>
-      <c r="I14" s="37" t="n"/>
-      <c r="J14" s="37" t="str">
+        <v>0.08290687209303722</v>
+      </c>
+      <c r="H14" s="37" t="n">
+        <v>13.98577139571209</v>
+      </c>
+      <c r="I14" s="37" t="n">
+        <v>20.73290581831791</v>
+      </c>
+      <c r="J14" s="37">
         <f>IF(AND(ISNUMBER(I14),ISNUMBER(H14)),I14-H14,"—")</f>
-        <v>—</v>
-      </c>
-      <c r="K14" s="31" t="n"/>
+        <v>6.74713442260582</v>
+      </c>
+      <c r="K14" s="31" t="n">
+        <v>0.01005870134701547</v>
+      </c>
       <c r="L14" s="50" t="str">
         <f>IF(AND(E14=3,E8=3),((B14&gt;B8)+(C14&gt;C8)+(D14&gt;D8))&amp;" of 3 folds","—")</f>
-        <v>—</v>
+        <v>1 of 3 folds</v>
       </c>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>not started yet</t>
+          <t>Mild overfitting</t>
         </is>
       </c>
     </row>
@@ -7986,35 +8034,47 @@
           <t>Bi-SRNet-lite + CE + rare sampling</t>
         </is>
       </c>
-      <c r="B15" s="41" t="n"/>
-      <c r="C15" s="41" t="n"/>
-      <c r="D15" s="41" t="n"/>
+      <c r="B15" s="41" t="n">
+        <v>13.33517132705466</v>
+      </c>
+      <c r="C15" s="41" t="n">
+        <v>13.2004769977504</v>
+      </c>
+      <c r="D15" s="41" t="n">
+        <v>13.36732759110079</v>
+      </c>
       <c r="E15" s="44">
         <f>COUNT(B15:D15)</f>
-        <v>0.0</v>
-      </c>
-      <c r="F15" s="41" t="str">
+        <v>3.0</v>
+      </c>
+      <c r="F15" s="41">
         <f>IF(E15&gt;0,AVERAGE(B15:D15),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="G15" s="41" t="str">
+        <v>13.300991971968616</v>
+      </c>
+      <c r="G15" s="41">
         <f>IF(E15&gt;1,STDEV(B15:D15),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="41" t="n"/>
-      <c r="J15" s="41" t="str">
+        <v>0.08852090917358249</v>
+      </c>
+      <c r="H15" s="41" t="n">
+        <v>13.88117494984814</v>
+      </c>
+      <c r="I15" s="41" t="n">
+        <v>22.37756728014341</v>
+      </c>
+      <c r="J15" s="41">
         <f>IF(AND(ISNUMBER(I15),ISNUMBER(H15)),I15-H15,"—")</f>
-        <v>—</v>
-      </c>
-      <c r="K15" s="33" t="n"/>
+        <v>8.49639233029527</v>
+      </c>
+      <c r="K15" s="33" t="n">
+        <v>0.01301278527036434</v>
+      </c>
       <c r="L15" s="54" t="str">
         <f>IF(AND(E15=3,E8=3),((B15&gt;B8)+(C15&gt;C8)+(D15&gt;D8))&amp;" of 3 folds","—")</f>
-        <v>—</v>
+        <v>1 of 3 folds</v>
       </c>
       <c r="M15" s="8" t="inlineStr">
         <is>
-          <t>not started yet</t>
+          <t>Mild overfitting</t>
         </is>
       </c>
     </row>
@@ -8024,35 +8084,47 @@
           <t>Bi-SRNet-lite + WCE + Dice + rare sampling</t>
         </is>
       </c>
-      <c r="B16" s="37" t="n"/>
-      <c r="C16" s="37" t="n"/>
-      <c r="D16" s="37" t="n"/>
+      <c r="B16" s="37" t="n">
+        <v>14.11677552568725</v>
+      </c>
+      <c r="C16" s="37" t="n">
+        <v>13.71763206610269</v>
+      </c>
+      <c r="D16" s="37" t="n">
+        <v>13.43770089023743</v>
+      </c>
       <c r="E16" s="40">
         <f>COUNT(B16:D16)</f>
-        <v>0.0</v>
-      </c>
-      <c r="F16" s="37" t="str">
+        <v>3.0</v>
+      </c>
+      <c r="F16" s="37">
         <f>IF(E16&gt;0,AVERAGE(B16:D16),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="G16" s="37" t="str">
+        <v>13.757369494009124</v>
+      </c>
+      <c r="G16" s="37">
         <f>IF(E16&gt;1,STDEV(B16:D16),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="H16" s="37" t="n"/>
-      <c r="I16" s="37" t="n"/>
-      <c r="J16" s="37" t="str">
+        <v>0.34127684877572784</v>
+      </c>
+      <c r="H16" s="37" t="n">
+        <v>14.52804886159683</v>
+      </c>
+      <c r="I16" s="37" t="n">
+        <v>23.0165563254746</v>
+      </c>
+      <c r="J16" s="37">
         <f>IF(AND(ISNUMBER(I16),ISNUMBER(H16)),I16-H16,"—")</f>
-        <v>—</v>
-      </c>
-      <c r="K16" s="31" t="n"/>
+        <v>8.48850746387777</v>
+      </c>
+      <c r="K16" s="31" t="n">
+        <v>0.01311934379824367</v>
+      </c>
       <c r="L16" s="50" t="str">
         <f>IF(AND(E16=3,E8=3),((B16&gt;B8)+(C16&gt;C8)+(D16&gt;D8))&amp;" of 3 folds","—")</f>
-        <v>—</v>
+        <v>3 of 3 folds</v>
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>not started yet</t>
+          <t>Mild overfitting</t>
         </is>
       </c>
     </row>
@@ -8062,35 +8134,47 @@
           <t>Bi-SRNet-lite + OHEM</t>
         </is>
       </c>
-      <c r="B17" s="41" t="n"/>
-      <c r="C17" s="41" t="n"/>
-      <c r="D17" s="41" t="n"/>
+      <c r="B17" s="41" t="n">
+        <v>3.016396692090735</v>
+      </c>
+      <c r="C17" s="41" t="n">
+        <v>3.482449335833063</v>
+      </c>
+      <c r="D17" s="41" t="n">
+        <v>3.523132357287033</v>
+      </c>
       <c r="E17" s="44">
         <f>COUNT(B17:D17)</f>
-        <v>0.0</v>
-      </c>
-      <c r="F17" s="41" t="str">
+        <v>3.0</v>
+      </c>
+      <c r="F17" s="41">
         <f>IF(E17&gt;0,AVERAGE(B17:D17),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="G17" s="41" t="str">
+        <v>3.340659461736944</v>
+      </c>
+      <c r="G17" s="41">
         <f>IF(E17&gt;1,STDEV(B17:D17),"—")</f>
-        <v>—</v>
-      </c>
-      <c r="H17" s="41" t="n"/>
-      <c r="I17" s="41" t="n"/>
-      <c r="J17" s="41" t="str">
+        <v>0.28155556270943877</v>
+      </c>
+      <c r="H17" s="41" t="n">
+        <v>3.327882838069222</v>
+      </c>
+      <c r="I17" s="41" t="n">
+        <v>4.525588847560931</v>
+      </c>
+      <c r="J17" s="41">
         <f>IF(AND(ISNUMBER(I17),ISNUMBER(H17)),I17-H17,"—")</f>
-        <v>—</v>
-      </c>
-      <c r="K17" s="33" t="n"/>
+        <v>1.197706009491709</v>
+      </c>
+      <c r="K17" s="33" t="n">
+        <v>0.002318960576435358</v>
+      </c>
       <c r="L17" s="54" t="str">
         <f>IF(AND(E17=3,E8=3),((B17&gt;B8)+(C17&gt;C8)+(D17&gt;D8))&amp;" of 3 folds","—")</f>
-        <v>—</v>
+        <v>0 of 3 folds</v>
       </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
-          <t>not started yet</t>
+          <t>Failed to learn</t>
         </is>
       </c>
     </row>
@@ -8120,6 +8204,8 @@
     <row r="37" ht="15" customHeight="1"/>
     <row r="38" ht="15" customHeight="1"/>
     <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
     <row r="42" ht="15" customHeight="1"/>
     <row r="43" ht="15" customHeight="1"/>
     <row r="44" ht="15" customHeight="1"/>
@@ -8127,8 +8213,6 @@
     <row r="46" ht="15" customHeight="1"/>
     <row r="47" ht="15" customHeight="1"/>
     <row r="48" ht="15" customHeight="1"/>
-    <row r="49" ht="15" customHeight="1"/>
-    <row r="50" ht="15" customHeight="1"/>
     <row r="51" ht="15" customHeight="1"/>
     <row r="52" ht="15" customHeight="1"/>
     <row r="53" ht="15" customHeight="1"/>
@@ -8138,523 +8222,1192 @@
     <row r="57" ht="15" customHeight="1"/>
     <row r="58" ht="15" customHeight="1"/>
     <row r="59" ht="15" customHeight="1"/>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="4" t="inlineStr">
+    <row r="60" ht="15" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="15" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1"/>
+    <row r="67" ht="15" customHeight="1"/>
+    <row r="68" ht="15" customHeight="1"/>
+    <row r="69" ht="15" customHeight="1"/>
+    <row r="70" ht="15" customHeight="1"/>
+    <row r="71" ht="15" customHeight="1"/>
+    <row r="72" ht="15" customHeight="1"/>
+    <row r="73" ht="15" customHeight="1"/>
+    <row r="74" ht="15" customHeight="1"/>
+    <row r="75" ht="15" customHeight="1"/>
+    <row r="76" ht="15" customHeight="1"/>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>Every fold in detail</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="35" customHeight="1">
-      <c r="A63" s="5" t="inlineStr">
+    <row r="81" ht="35" customHeight="1">
+      <c r="A81" s="5" t="inlineStr">
         <is>
           <t>Configuration</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B81" s="5" t="inlineStr">
         <is>
           <t>Fold</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>Best epoch</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="D81" s="5" t="inlineStr">
         <is>
           <t>Train SeK</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
+      <c r="E81" s="5" t="inlineStr">
         <is>
           <t>Val SeK</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr">
+      <c r="F81" s="5" t="inlineStr">
         <is>
           <t>Test SeK</t>
         </is>
       </c>
-      <c r="G63" s="5" t="inlineStr">
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>Test Fscd</t>
         </is>
       </c>
-      <c r="H63" s="5" t="inlineStr">
+      <c r="H81" s="5" t="inlineStr">
         <is>
           <t>Test mIoU</t>
         </is>
       </c>
-      <c r="I63" s="5" t="inlineStr">
+      <c r="I81" s="5" t="inlineStr">
         <is>
           <t>Test OA</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="18.5" customHeight="1">
-      <c r="A64" s="6" t="inlineStr">
+    <row r="82" ht="18.5" customHeight="1">
+      <c r="A82" s="6" t="inlineStr">
         <is>
           <t>Early Fusion + CE (baseline)</t>
         </is>
       </c>
-      <c r="B64" s="40" t="n">
+      <c r="B82" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C64" s="40" t="n">
+      <c r="C82" s="40" t="n">
         <v>17</v>
       </c>
-      <c r="D64" s="37" t="n">
+      <c r="D82" s="37" t="n">
         <v>11.652523953531</v>
       </c>
-      <c r="E64" s="37" t="n">
+      <c r="E82" s="37" t="n">
         <v>6.737039572166093</v>
       </c>
-      <c r="F64" s="37" t="n">
+      <c r="F82" s="37" t="n">
         <v>6.645246316795617</v>
       </c>
-      <c r="G64" s="37" t="n">
+      <c r="G82" s="37" t="n">
         <v>43.72996682761042</v>
       </c>
-      <c r="H64" s="37" t="n">
+      <c r="H82" s="37" t="n">
         <v>62.4234713916467</v>
       </c>
-      <c r="I64" s="37" t="n">
+      <c r="I82" s="37" t="n">
         <v>84.02053448332458</v>
       </c>
     </row>
-    <row r="65" ht="18.5" customHeight="1">
-      <c r="A65" s="8" t="inlineStr">
+    <row r="83" ht="18.5" customHeight="1">
+      <c r="A83" s="8" t="inlineStr">
         <is>
           <t>Early Fusion + CE (baseline)</t>
         </is>
       </c>
-      <c r="B65" s="44" t="n">
+      <c r="B83" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="C65" s="44" t="n">
+      <c r="C83" s="44" t="n">
         <v>18</v>
       </c>
-      <c r="D65" s="41" t="n">
+      <c r="D83" s="41" t="n">
         <v>12.20344207102451</v>
       </c>
-      <c r="E65" s="41" t="n">
+      <c r="E83" s="41" t="n">
         <v>7.073141991388574</v>
       </c>
-      <c r="F65" s="41" t="n">
+      <c r="F83" s="41" t="n">
         <v>6.774199408087096</v>
       </c>
-      <c r="G65" s="41" t="n">
+      <c r="G83" s="41" t="n">
         <v>44.98113162695889</v>
       </c>
-      <c r="H65" s="41" t="n">
+      <c r="H83" s="41" t="n">
         <v>62.99649592299038</v>
       </c>
-      <c r="I65" s="41" t="n">
+      <c r="I83" s="41" t="n">
         <v>83.41428099560136</v>
       </c>
     </row>
-    <row r="66" ht="18.5" customHeight="1">
-      <c r="A66" s="6" t="inlineStr">
+    <row r="84" ht="18.5" customHeight="1">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>Early Fusion + CE (baseline)</t>
         </is>
       </c>
-      <c r="B66" s="40" t="n">
+      <c r="B84" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="C66" s="40" t="n">
+      <c r="C84" s="40" t="n">
         <v>15</v>
       </c>
-      <c r="D66" s="37" t="n">
+      <c r="D84" s="37" t="n">
         <v>11.48805131631928</v>
       </c>
-      <c r="E66" s="37" t="n">
+      <c r="E84" s="37" t="n">
         <v>7.292101446957481</v>
       </c>
-      <c r="F66" s="37" t="n">
+      <c r="F84" s="37" t="n">
         <v>6.815470927609538</v>
       </c>
-      <c r="G66" s="37" t="n">
+      <c r="G84" s="37" t="n">
         <v>44.61715350687294</v>
       </c>
-      <c r="H66" s="37" t="n">
+      <c r="H84" s="37" t="n">
         <v>62.93391071291344</v>
       </c>
-      <c r="I66" s="37" t="n">
+      <c r="I84" s="37" t="n">
         <v>83.64949971687894</v>
       </c>
     </row>
-    <row r="67" ht="18.5" customHeight="1">
-      <c r="A67" s="8" t="inlineStr">
+    <row r="85" ht="18.5" customHeight="1">
+      <c r="A85" s="8" t="inlineStr">
         <is>
           <t>SSCD + CE (baseline)</t>
         </is>
       </c>
-      <c r="B67" s="44" t="n">
+      <c r="B85" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="C67" s="44" t="n">
+      <c r="C85" s="44" t="n">
         <v>20</v>
       </c>
-      <c r="D67" s="41" t="n">
+      <c r="D85" s="41" t="n">
         <v>25.20596867822439</v>
       </c>
-      <c r="E67" s="41" t="n">
+      <c r="E85" s="41" t="n">
         <v>13.54996647520109</v>
       </c>
-      <c r="F67" s="41" t="n">
+      <c r="F85" s="41" t="n">
         <v>13.38600274344059</v>
       </c>
-      <c r="G67" s="41" t="n">
+      <c r="G85" s="41" t="n">
         <v>52.14881930331633</v>
       </c>
-      <c r="H67" s="41" t="n">
+      <c r="H85" s="41" t="n">
         <v>68.10464105376413</v>
       </c>
-      <c r="I67" s="41" t="n">
+      <c r="I85" s="41" t="n">
         <v>85.89617304441308</v>
       </c>
     </row>
-    <row r="68" ht="18.5" customHeight="1">
-      <c r="A68" s="6" t="inlineStr">
+    <row r="86" ht="18.5" customHeight="1">
+      <c r="A86" s="6" t="inlineStr">
         <is>
           <t>SSCD + CE (baseline)</t>
         </is>
       </c>
-      <c r="B68" s="40" t="n">
+      <c r="B86" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="C68" s="40" t="n">
+      <c r="C86" s="40" t="n">
         <v>20</v>
       </c>
-      <c r="D68" s="37" t="n">
+      <c r="D86" s="37" t="n">
         <v>24.97820983396715</v>
       </c>
-      <c r="E68" s="37" t="n">
+      <c r="E86" s="37" t="n">
         <v>12.57441935370468</v>
       </c>
-      <c r="F68" s="37" t="n">
+      <c r="F86" s="37" t="n">
         <v>12.91766336066057</v>
       </c>
-      <c r="G68" s="37" t="n">
+      <c r="G86" s="37" t="n">
         <v>51.71308270071261</v>
       </c>
-      <c r="H68" s="37" t="n">
+      <c r="H86" s="37" t="n">
         <v>67.67203569838581</v>
       </c>
-      <c r="I68" s="37" t="n">
+      <c r="I86" s="37" t="n">
         <v>85.67207528763458</v>
       </c>
     </row>
-    <row r="69" ht="18.5" customHeight="1">
-      <c r="A69" s="8" t="inlineStr">
+    <row r="87" ht="18.5" customHeight="1">
+      <c r="A87" s="8" t="inlineStr">
         <is>
           <t>SSCD + CE (baseline)</t>
         </is>
       </c>
-      <c r="B69" s="44" t="n">
+      <c r="B87" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="C69" s="44" t="n">
+      <c r="C87" s="44" t="n">
         <v>20</v>
       </c>
-      <c r="D69" s="41" t="n">
+      <c r="D87" s="41" t="n">
         <v>25.33617929840592</v>
       </c>
-      <c r="E69" s="41" t="n">
+      <c r="E87" s="41" t="n">
         <v>14.0046642651508</v>
       </c>
-      <c r="F69" s="41" t="n">
+      <c r="F87" s="41" t="n">
         <v>12.61108932305377</v>
       </c>
-      <c r="G69" s="41" t="n">
+      <c r="G87" s="41" t="n">
         <v>51.15124398317518</v>
       </c>
-      <c r="H69" s="41" t="n">
+      <c r="H87" s="41" t="n">
         <v>67.46508915278571</v>
       </c>
-      <c r="I69" s="41" t="n">
+      <c r="I87" s="41" t="n">
         <v>85.64202444893974</v>
       </c>
     </row>
-    <row r="70" ht="18.5" customHeight="1">
-      <c r="A70" s="6" t="inlineStr">
+    <row r="88" ht="18.5" customHeight="1">
+      <c r="A88" s="6" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + CE (baseline)</t>
         </is>
       </c>
-      <c r="B70" s="40" t="n">
+      <c r="B88" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C70" s="40" t="n">
+      <c r="C88" s="40" t="n">
         <v>20</v>
       </c>
-      <c r="D70" s="37" t="n">
+      <c r="D88" s="37" t="n">
         <v>23.7853273704451</v>
       </c>
-      <c r="E70" s="37" t="n">
+      <c r="E88" s="37" t="n">
         <v>14.65933526551606</v>
       </c>
-      <c r="F70" s="37" t="n">
+      <c r="F88" s="37" t="n">
         <v>14.003732339286</v>
       </c>
-      <c r="G70" s="37" t="n">
+      <c r="G88" s="37" t="n">
         <v>53.26246703573447</v>
       </c>
-      <c r="H70" s="37" t="n">
+      <c r="H88" s="37" t="n">
         <v>68.30146426164599</v>
       </c>
-      <c r="I70" s="37" t="n">
+      <c r="I88" s="37" t="n">
         <v>85.97268497242648</v>
       </c>
     </row>
-    <row r="71" ht="18.5" customHeight="1">
-      <c r="A71" s="8" t="inlineStr">
+    <row r="89" ht="18.5" customHeight="1">
+      <c r="A89" s="8" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + CE (baseline)</t>
         </is>
       </c>
-      <c r="B71" s="44" t="n">
+      <c r="B89" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="C71" s="44" t="n">
+      <c r="C89" s="44" t="n">
         <v>14</v>
       </c>
-      <c r="D71" s="41" t="n">
+      <c r="D89" s="41" t="n">
         <v>21.97265668535853</v>
       </c>
-      <c r="E71" s="41" t="n">
+      <c r="E89" s="41" t="n">
         <v>13.76819145345096</v>
       </c>
-      <c r="F71" s="41" t="n">
+      <c r="F89" s="41" t="n">
         <v>13.49485020581882</v>
       </c>
-      <c r="G71" s="41" t="n">
+      <c r="G89" s="41" t="n">
         <v>52.8720836243621</v>
       </c>
-      <c r="H71" s="41" t="n">
+      <c r="H89" s="41" t="n">
         <v>67.89658443962358</v>
       </c>
-      <c r="I71" s="41" t="n">
+      <c r="I89" s="41" t="n">
         <v>85.62856978728992</v>
       </c>
     </row>
-    <row r="72" ht="18.5" customHeight="1">
-      <c r="A72" s="6" t="inlineStr">
+    <row r="90" ht="18.5" customHeight="1">
+      <c r="A90" s="6" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + CE (baseline)</t>
         </is>
       </c>
-      <c r="B72" s="40" t="n">
+      <c r="B90" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="C72" s="40" t="n">
+      <c r="C90" s="40" t="n">
         <v>20</v>
       </c>
-      <c r="D72" s="37" t="n">
+      <c r="D90" s="37" t="n">
         <v>23.72314331211742</v>
       </c>
-      <c r="E72" s="37" t="n">
+      <c r="E90" s="37" t="n">
         <v>14.74593431011282</v>
       </c>
-      <c r="F72" s="37" t="n">
+      <c r="F90" s="37" t="n">
         <v>13.16045465382735</v>
       </c>
-      <c r="G72" s="37" t="n">
+      <c r="G90" s="37" t="n">
         <v>52.22949669023814</v>
       </c>
-      <c r="H72" s="37" t="n">
+      <c r="H90" s="37" t="n">
         <v>67.56676186056923</v>
       </c>
-      <c r="I72" s="37" t="n">
+      <c r="I90" s="37" t="n">
         <v>85.75758861894367</v>
       </c>
     </row>
-    <row r="73" ht="18.5" customHeight="1">
-      <c r="A73" s="8" t="inlineStr">
+    <row r="91" ht="18.5" customHeight="1">
+      <c r="A91" s="8" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + WCE + Dice</t>
         </is>
       </c>
-      <c r="B73" s="44" t="n">
+      <c r="B91" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="C73" s="44" t="n">
+      <c r="C91" s="44" t="n">
         <v>20</v>
       </c>
-      <c r="D73" s="41" t="n">
+      <c r="D91" s="41" t="n">
         <v>23.92941948315633</v>
       </c>
-      <c r="E73" s="41" t="n">
+      <c r="E91" s="41" t="n">
         <v>15.20032450528961</v>
       </c>
-      <c r="F73" s="41" t="n">
+      <c r="F91" s="41" t="n">
         <v>14.46719244575141</v>
       </c>
-      <c r="G73" s="41" t="n">
+      <c r="G91" s="41" t="n">
         <v>53.05288539416152</v>
       </c>
-      <c r="H73" s="41" t="n">
+      <c r="H91" s="41" t="n">
         <v>68.45048879451983</v>
       </c>
-      <c r="I73" s="41" t="n">
+      <c r="I91" s="41" t="n">
         <v>83.8690108611804</v>
       </c>
     </row>
-    <row r="74" ht="18.5" customHeight="1">
-      <c r="A74" s="6" t="inlineStr">
+    <row r="92" ht="18.5" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + WCE + Dice</t>
         </is>
       </c>
-      <c r="B74" s="40" t="n">
+      <c r="B92" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="C74" s="40" t="n">
+      <c r="C92" s="40" t="n">
         <v>20</v>
       </c>
-      <c r="D74" s="37" t="n">
+      <c r="D92" s="37" t="n">
         <v>23.41410242374137</v>
       </c>
-      <c r="E74" s="37" t="n">
+      <c r="E92" s="37" t="n">
         <v>14.2554344600486</v>
       </c>
-      <c r="F74" s="37" t="n">
+      <c r="F92" s="37" t="n">
         <v>14.10384023694363</v>
       </c>
-      <c r="G74" s="37" t="n">
+      <c r="G92" s="37" t="n">
         <v>52.65863904669897</v>
       </c>
-      <c r="H74" s="37" t="n">
+      <c r="H92" s="37" t="n">
         <v>68.12598590569634</v>
       </c>
-      <c r="I74" s="37" t="n">
+      <c r="I92" s="37" t="n">
         <v>83.72648479557839</v>
       </c>
     </row>
-    <row r="75" ht="18.5" customHeight="1">
-      <c r="A75" s="8" t="inlineStr">
+    <row r="93" ht="18.5" customHeight="1">
+      <c r="A93" s="8" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + WCE + Dice</t>
         </is>
       </c>
-      <c r="B75" s="44" t="n">
+      <c r="B93" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="C75" s="44" t="n">
+      <c r="C93" s="44" t="n">
         <v>20</v>
       </c>
-      <c r="D75" s="41" t="n">
+      <c r="D93" s="41" t="n">
         <v>25.19073776549882</v>
       </c>
-      <c r="E75" s="41" t="n">
+      <c r="E93" s="41" t="n">
         <v>15.42509701081625</v>
       </c>
-      <c r="F75" s="41" t="n">
+      <c r="F93" s="41" t="n">
         <v>14.19617163288387</v>
       </c>
-      <c r="G75" s="41" t="n">
+      <c r="G93" s="41" t="n">
         <v>52.60091238990265</v>
       </c>
-      <c r="H75" s="41" t="n">
+      <c r="H93" s="41" t="n">
         <v>68.14776821074608</v>
       </c>
-      <c r="I75" s="41" t="n">
+      <c r="I93" s="41" t="n">
         <v>83.68453979492188</v>
       </c>
     </row>
-    <row r="76" ht="18.5" customHeight="1">
-      <c r="A76" s="6" t="inlineStr">
+    <row r="94" ht="18.5" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + CE + Dice</t>
         </is>
       </c>
-      <c r="B76" s="40" t="n">
+      <c r="B94" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C76" s="40" t="n">
+      <c r="C94" s="40" t="n">
         <v>20</v>
       </c>
-      <c r="D76" s="37" t="n">
+      <c r="D94" s="37" t="n">
         <v>23.92965121602546</v>
       </c>
-      <c r="E76" s="37" t="n">
+      <c r="E94" s="37" t="n">
         <v>15.44304421585181</v>
       </c>
-      <c r="F76" s="37" t="n">
+      <c r="F94" s="37" t="n">
         <v>14.73100366812015</v>
       </c>
-      <c r="G76" s="37" t="n">
+      <c r="G94" s="37" t="n">
         <v>54.15697224513754</v>
       </c>
-      <c r="H76" s="37" t="n">
+      <c r="H94" s="37" t="n">
         <v>68.8531115506228</v>
       </c>
-      <c r="I76" s="37" t="n">
+      <c r="I94" s="37" t="n">
         <v>85.28636130966059</v>
       </c>
     </row>
-    <row r="77" ht="18.5" customHeight="1">
-      <c r="A77" s="8" t="inlineStr">
+    <row r="95" ht="18.5" customHeight="1">
+      <c r="A95" s="8" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + CE + Dice</t>
         </is>
       </c>
-      <c r="B77" s="44" t="n">
+      <c r="B95" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="C77" s="44" t="n">
+      <c r="C95" s="44" t="n">
         <v>20</v>
       </c>
-      <c r="D77" s="41" t="n">
+      <c r="D95" s="41" t="n">
         <v>24.20779154751237</v>
       </c>
-      <c r="E77" s="41" t="n">
+      <c r="E95" s="41" t="n">
         <v>13.95965071837446</v>
       </c>
-      <c r="F77" s="41" t="n">
+      <c r="F95" s="41" t="n">
         <v>14.17122852987455</v>
       </c>
-      <c r="G77" s="41" t="n">
+      <c r="G95" s="41" t="n">
         <v>53.40367925079037</v>
       </c>
-      <c r="H77" s="41" t="n">
+      <c r="H95" s="41" t="n">
         <v>68.63482047748732</v>
       </c>
-      <c r="I77" s="41" t="n">
+      <c r="I95" s="41" t="n">
         <v>85.15293666294643</v>
       </c>
     </row>
-    <row r="78" ht="18.5" customHeight="1">
-      <c r="A78" s="6" t="inlineStr">
+    <row r="96" ht="18.5" customHeight="1">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>Bi-SRNet-lite + CE + Dice</t>
         </is>
       </c>
-      <c r="B78" s="40" t="n">
+      <c r="B96" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="C78" s="40" t="n">
+      <c r="C96" s="40" t="n">
         <v>20</v>
       </c>
-      <c r="D78" s="37" t="n">
+      <c r="D96" s="37" t="n">
         <v>25.39178152584292</v>
       </c>
-      <c r="E78" s="37" t="n">
+      <c r="E96" s="37" t="n">
         <v>15.51828246757415</v>
       </c>
-      <c r="F78" s="37" t="n">
+      <c r="F96" s="37" t="n">
         <v>14.23387451645121</v>
       </c>
-      <c r="G78" s="37" t="n">
+      <c r="G96" s="37" t="n">
         <v>53.48052447775882</v>
       </c>
-      <c r="H78" s="37" t="n">
+      <c r="H96" s="37" t="n">
         <v>68.59749169714989</v>
       </c>
-      <c r="I78" s="37" t="n">
+      <c r="I96" s="37" t="n">
         <v>85.25599119042148</v>
+      </c>
+    </row>
+    <row r="97" ht="18.5" customHeight="1">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Weighted CE</t>
+        </is>
+      </c>
+      <c r="B97" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C97" s="44" t="n">
+        <v>20</v>
+      </c>
+      <c r="D97" s="41" t="n">
+        <v>23.47453018856701</v>
+      </c>
+      <c r="E97" s="41" t="n">
+        <v>15.08217692109497</v>
+      </c>
+      <c r="F97" s="41" t="n">
+        <v>14.64664541715592</v>
+      </c>
+      <c r="G97" s="41" t="n">
+        <v>53.21326189890915</v>
+      </c>
+      <c r="H97" s="41" t="n">
+        <v>68.56230410394379</v>
+      </c>
+      <c r="I97" s="41" t="n">
+        <v>83.94457007656578</v>
+      </c>
+    </row>
+    <row r="98" ht="18.5" customHeight="1">
+      <c r="A98" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Weighted CE</t>
+        </is>
+      </c>
+      <c r="B98" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C98" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="D98" s="37" t="n">
+        <v>22.2232863804846</v>
+      </c>
+      <c r="E98" s="37" t="n">
+        <v>14.26470555871296</v>
+      </c>
+      <c r="F98" s="37" t="n">
+        <v>14.26148333562495</v>
+      </c>
+      <c r="G98" s="37" t="n">
+        <v>52.8782137248562</v>
+      </c>
+      <c r="H98" s="37" t="n">
+        <v>68.12726730395546</v>
+      </c>
+      <c r="I98" s="37" t="n">
+        <v>83.74132557075565</v>
+      </c>
+    </row>
+    <row r="99" ht="18.5" customHeight="1">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Weighted CE</t>
+        </is>
+      </c>
+      <c r="B99" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C99" s="44" t="n">
+        <v>20</v>
+      </c>
+      <c r="D99" s="41" t="n">
+        <v>23.14470497542326</v>
+      </c>
+      <c r="E99" s="41" t="n">
+        <v>15.31544406483176</v>
+      </c>
+      <c r="F99" s="41" t="n">
+        <v>14.14211735890099</v>
+      </c>
+      <c r="G99" s="41" t="n">
+        <v>52.59946515526713</v>
+      </c>
+      <c r="H99" s="41" t="n">
+        <v>67.98973540544414</v>
+      </c>
+      <c r="I99" s="41" t="n">
+        <v>83.66017189346442</v>
+      </c>
+    </row>
+    <row r="100" ht="18.5" customHeight="1">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Median-freq</t>
+        </is>
+      </c>
+      <c r="B100" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C100" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="D100" s="37" t="n">
+        <v>20.91301808999058</v>
+      </c>
+      <c r="E100" s="37" t="n">
+        <v>14.67650547265047</v>
+      </c>
+      <c r="F100" s="37" t="n">
+        <v>14.20669732292025</v>
+      </c>
+      <c r="G100" s="37" t="n">
+        <v>52.11183509519126</v>
+      </c>
+      <c r="H100" s="37" t="n">
+        <v>68.26686565286661</v>
+      </c>
+      <c r="I100" s="37" t="n">
+        <v>83.55806494961266</v>
+      </c>
+    </row>
+    <row r="101" ht="18.5" customHeight="1">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Median-freq</t>
+        </is>
+      </c>
+      <c r="B101" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C101" s="44" t="n">
+        <v>19</v>
+      </c>
+      <c r="D101" s="41" t="n">
+        <v>20.50913351048096</v>
+      </c>
+      <c r="E101" s="41" t="n">
+        <v>13.70765414113065</v>
+      </c>
+      <c r="F101" s="41" t="n">
+        <v>13.56942910926994</v>
+      </c>
+      <c r="G101" s="41" t="n">
+        <v>51.35247766377908</v>
+      </c>
+      <c r="H101" s="41" t="n">
+        <v>68.23660436332753</v>
+      </c>
+      <c r="I101" s="41" t="n">
+        <v>83.71941061580883</v>
+      </c>
+    </row>
+    <row r="102" ht="18.5" customHeight="1">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Median-freq</t>
+        </is>
+      </c>
+      <c r="B102" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C102" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="D102" s="37" t="n">
+        <v>21.5772206955468</v>
+      </c>
+      <c r="E102" s="37" t="n">
+        <v>14.8015812648764</v>
+      </c>
+      <c r="F102" s="37" t="n">
+        <v>13.4191390301541</v>
+      </c>
+      <c r="G102" s="37" t="n">
+        <v>50.92109133328264</v>
+      </c>
+      <c r="H102" s="37" t="n">
+        <v>67.83204567715842</v>
+      </c>
+      <c r="I102" s="37" t="n">
+        <v>83.29569071280855</v>
+      </c>
+    </row>
+    <row r="103" ht="18.5" customHeight="1">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Class-balanced</t>
+        </is>
+      </c>
+      <c r="B103" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C103" s="44" t="n">
+        <v>20</v>
+      </c>
+      <c r="D103" s="41" t="n">
+        <v>22.36033182160223</v>
+      </c>
+      <c r="E103" s="41" t="n">
+        <v>14.9740448149722</v>
+      </c>
+      <c r="F103" s="41" t="n">
+        <v>14.37406026945466</v>
+      </c>
+      <c r="G103" s="41" t="n">
+        <v>52.59771104215184</v>
+      </c>
+      <c r="H103" s="41" t="n">
+        <v>68.43811026261557</v>
+      </c>
+      <c r="I103" s="41" t="n">
+        <v>83.68713891806723</v>
+      </c>
+    </row>
+    <row r="104" ht="18.5" customHeight="1">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Class-balanced</t>
+        </is>
+      </c>
+      <c r="B104" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C104" s="40" t="n">
+        <v>17</v>
+      </c>
+      <c r="D104" s="37" t="n">
+        <v>21.42981107771852</v>
+      </c>
+      <c r="E104" s="37" t="n">
+        <v>13.98865176340754</v>
+      </c>
+      <c r="F104" s="37" t="n">
+        <v>14.38428715583249</v>
+      </c>
+      <c r="G104" s="37" t="n">
+        <v>52.95050664465796</v>
+      </c>
+      <c r="H104" s="37" t="n">
+        <v>68.63607822346684</v>
+      </c>
+      <c r="I104" s="37" t="n">
+        <v>84.53887811228007</v>
+      </c>
+    </row>
+    <row r="105" ht="18.5" customHeight="1">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Class-balanced</t>
+        </is>
+      </c>
+      <c r="B105" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C105" s="44" t="n">
+        <v>20</v>
+      </c>
+      <c r="D105" s="41" t="n">
+        <v>22.49123319837551</v>
+      </c>
+      <c r="E105" s="41" t="n">
+        <v>15.2791202964545</v>
+      </c>
+      <c r="F105" s="41" t="n">
+        <v>13.68703818601729</v>
+      </c>
+      <c r="G105" s="41" t="n">
+        <v>51.84184658203207</v>
+      </c>
+      <c r="H105" s="41" t="n">
+        <v>67.85521643235516</v>
+      </c>
+      <c r="I105" s="41" t="n">
+        <v>83.46859202665441</v>
+      </c>
+    </row>
+    <row r="106" ht="18.5" customHeight="1">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Focal</t>
+        </is>
+      </c>
+      <c r="B106" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C106" s="40" t="n">
+        <v>17</v>
+      </c>
+      <c r="D106" s="37" t="n">
+        <v>20.42834765407203</v>
+      </c>
+      <c r="E106" s="37" t="n">
+        <v>14.35678614324822</v>
+      </c>
+      <c r="F106" s="37" t="n">
+        <v>13.34032062207497</v>
+      </c>
+      <c r="G106" s="37" t="n">
+        <v>52.01355833203569</v>
+      </c>
+      <c r="H106" s="37" t="n">
+        <v>66.7851251120523</v>
+      </c>
+      <c r="I106" s="37" t="n">
+        <v>82.33047741801799</v>
+      </c>
+    </row>
+    <row r="107" ht="18.5" customHeight="1">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Focal</t>
+        </is>
+      </c>
+      <c r="B107" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C107" s="44" t="n">
+        <v>17</v>
+      </c>
+      <c r="D107" s="41" t="n">
+        <v>21.06070511839584</v>
+      </c>
+      <c r="E107" s="41" t="n">
+        <v>13.39745123436186</v>
+      </c>
+      <c r="F107" s="41" t="n">
+        <v>13.43639077930197</v>
+      </c>
+      <c r="G107" s="41" t="n">
+        <v>52.00338803237453</v>
+      </c>
+      <c r="H107" s="41" t="n">
+        <v>66.91957090129219</v>
+      </c>
+      <c r="I107" s="41" t="n">
+        <v>82.43227533933495</v>
+      </c>
+    </row>
+    <row r="108" ht="18.5" customHeight="1">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + Focal</t>
+        </is>
+      </c>
+      <c r="B108" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C108" s="40" t="n">
+        <v>17</v>
+      </c>
+      <c r="D108" s="37" t="n">
+        <v>20.70966468248586</v>
+      </c>
+      <c r="E108" s="37" t="n">
+        <v>14.20307680952619</v>
+      </c>
+      <c r="F108" s="37" t="n">
+        <v>13.27131493006328</v>
+      </c>
+      <c r="G108" s="37" t="n">
+        <v>51.61947031765337</v>
+      </c>
+      <c r="H108" s="37" t="n">
+        <v>66.33586674754007</v>
+      </c>
+      <c r="I108" s="37" t="n">
+        <v>81.93166780872505</v>
+      </c>
+    </row>
+    <row r="109" ht="18.5" customHeight="1">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + CE + rare sampling</t>
+        </is>
+      </c>
+      <c r="B109" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C109" s="44" t="n">
+        <v>19</v>
+      </c>
+      <c r="D109" s="41" t="n">
+        <v>23.15891762573616</v>
+      </c>
+      <c r="E109" s="41" t="n">
+        <v>13.81775622672125</v>
+      </c>
+      <c r="F109" s="41" t="n">
+        <v>13.33517132705466</v>
+      </c>
+      <c r="G109" s="41" t="n">
+        <v>52.33896230626538</v>
+      </c>
+      <c r="H109" s="41" t="n">
+        <v>67.77716776540711</v>
+      </c>
+      <c r="I109" s="41" t="n">
+        <v>85.82137548622964</v>
+      </c>
+    </row>
+    <row r="110" ht="18.5" customHeight="1">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + CE + rare sampling</t>
+        </is>
+      </c>
+      <c r="B110" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C110" s="40" t="n">
+        <v>19</v>
+      </c>
+      <c r="D110" s="37" t="n">
+        <v>21.71946335222322</v>
+      </c>
+      <c r="E110" s="37" t="n">
+        <v>13.17559994968464</v>
+      </c>
+      <c r="F110" s="37" t="n">
+        <v>13.2004769977504</v>
+      </c>
+      <c r="G110" s="37" t="n">
+        <v>52.29286974146657</v>
+      </c>
+      <c r="H110" s="37" t="n">
+        <v>67.73957689267567</v>
+      </c>
+      <c r="I110" s="37" t="n">
+        <v>85.70250439042805</v>
+      </c>
+    </row>
+    <row r="111" ht="18.5" customHeight="1">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + CE + rare sampling</t>
+        </is>
+      </c>
+      <c r="B111" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C111" s="44" t="n">
+        <v>16</v>
+      </c>
+      <c r="D111" s="41" t="n">
+        <v>22.25432086247087</v>
+      </c>
+      <c r="E111" s="41" t="n">
+        <v>14.65016867313855</v>
+      </c>
+      <c r="F111" s="41" t="n">
+        <v>13.36732759110079</v>
+      </c>
+      <c r="G111" s="41" t="n">
+        <v>52.74709583578001</v>
+      </c>
+      <c r="H111" s="41" t="n">
+        <v>67.89315288271753</v>
+      </c>
+      <c r="I111" s="41" t="n">
+        <v>85.15650773248753</v>
+      </c>
+    </row>
+    <row r="112" ht="32" customHeight="1">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + WCE + Dice + rare sampling</t>
+        </is>
+      </c>
+      <c r="B112" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C112" s="40" t="n">
+        <v>17</v>
+      </c>
+      <c r="D112" s="37" t="n">
+        <v>23.41691759028638</v>
+      </c>
+      <c r="E112" s="37" t="n">
+        <v>14.92927382726819</v>
+      </c>
+      <c r="F112" s="37" t="n">
+        <v>14.11677552568725</v>
+      </c>
+      <c r="G112" s="37" t="n">
+        <v>52.99174665815567</v>
+      </c>
+      <c r="H112" s="37" t="n">
+        <v>68.25648794353469</v>
+      </c>
+      <c r="I112" s="37" t="n">
+        <v>84.17499317842372</v>
+      </c>
+    </row>
+    <row r="113" ht="32" customHeight="1">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + WCE + Dice + rare sampling</t>
+        </is>
+      </c>
+      <c r="B113" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C113" s="44" t="n">
+        <v>19</v>
+      </c>
+      <c r="D113" s="41" t="n">
+        <v>22.34277876215799</v>
+      </c>
+      <c r="E113" s="41" t="n">
+        <v>13.98115634384826</v>
+      </c>
+      <c r="F113" s="41" t="n">
+        <v>13.71763206610269</v>
+      </c>
+      <c r="G113" s="41" t="n">
+        <v>52.20426848794993</v>
+      </c>
+      <c r="H113" s="41" t="n">
+        <v>67.98387707140864</v>
+      </c>
+      <c r="I113" s="41" t="n">
+        <v>83.68492190577402</v>
+      </c>
+    </row>
+    <row r="114" ht="32" customHeight="1">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + WCE + Dice + rare sampling</t>
+        </is>
+      </c>
+      <c r="B114" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C114" s="40" t="n">
+        <v>19</v>
+      </c>
+      <c r="D114" s="37" t="n">
+        <v>23.28997262397942</v>
+      </c>
+      <c r="E114" s="37" t="n">
+        <v>14.67371641367406</v>
+      </c>
+      <c r="F114" s="37" t="n">
+        <v>13.43770089023743</v>
+      </c>
+      <c r="G114" s="37" t="n">
+        <v>51.68635347272716</v>
+      </c>
+      <c r="H114" s="37" t="n">
+        <v>67.48406279704612</v>
+      </c>
+      <c r="I114" s="37" t="n">
+        <v>83.17988035057773</v>
+      </c>
+    </row>
+    <row r="115" ht="18.5" customHeight="1">
+      <c r="A115" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + OHEM</t>
+        </is>
+      </c>
+      <c r="B115" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C115" s="44" t="n">
+        <v>20</v>
+      </c>
+      <c r="D115" s="41" t="n">
+        <v>4.394526614825421</v>
+      </c>
+      <c r="E115" s="41" t="n">
+        <v>2.738701047679539</v>
+      </c>
+      <c r="F115" s="41" t="n">
+        <v>3.016396692090735</v>
+      </c>
+      <c r="G115" s="41" t="n">
+        <v>39.76620006069476</v>
+      </c>
+      <c r="H115" s="41" t="n">
+        <v>59.88675810962751</v>
+      </c>
+      <c r="I115" s="41" t="n">
+        <v>80.90845829298516</v>
+      </c>
+    </row>
+    <row r="116" ht="18.5" customHeight="1">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + OHEM</t>
+        </is>
+      </c>
+      <c r="B116" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C116" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="D116" s="37" t="n">
+        <v>4.497736629295048</v>
+      </c>
+      <c r="E116" s="37" t="n">
+        <v>3.39413682977816</v>
+      </c>
+      <c r="F116" s="37" t="n">
+        <v>3.482449335833063</v>
+      </c>
+      <c r="G116" s="37" t="n">
+        <v>31.55652451882116</v>
+      </c>
+      <c r="H116" s="37" t="n">
+        <v>44.40113180524185</v>
+      </c>
+      <c r="I116" s="37" t="n">
+        <v>59.38412321715796</v>
+      </c>
+    </row>
+    <row r="117" ht="18.5" customHeight="1">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t>Bi-SRNet-lite + OHEM</t>
+        </is>
+      </c>
+      <c r="B117" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C117" s="44" t="n">
+        <v>17</v>
+      </c>
+      <c r="D117" s="41" t="n">
+        <v>4.684503298562325</v>
+      </c>
+      <c r="E117" s="41" t="n">
+        <v>3.850810636749965</v>
+      </c>
+      <c r="F117" s="41" t="n">
+        <v>3.523132357287033</v>
+      </c>
+      <c r="G117" s="41" t="n">
+        <v>29.82686292562423</v>
+      </c>
+      <c r="H117" s="41" t="n">
+        <v>39.86695583182444</v>
+      </c>
+      <c r="I117" s="41" t="n">
+        <v>53.78817646443343</v>
       </c>
     </row>
   </sheetData>
@@ -8677,7 +9430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:Y102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8692,6 +9445,19 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.6" customHeight="1">
@@ -8711,7 +9477,7 @@
     <row r="3" ht="35.7" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Key takeaway: So far: 5 × mild overfitting. The validation score flattens after about 12–15 epochs while the training score keeps rising, so longer training alone is unlikely to help much.</t>
+          <t>Key takeaway: 11 × mild overfitting, 1 × failed to learn. In every configuration the training score keeps rising while the validation score grows only slowly after about 12–15 epochs. More data or regularisation should help more than simply training longer.</t>
         </is>
       </c>
     </row>
@@ -8737,6 +9503,8 @@
     <row r="24" ht="15" customHeight="1"/>
     <row r="25" ht="15" customHeight="1"/>
     <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
     <row r="29" ht="15" customHeight="1"/>
     <row r="30" ht="15" customHeight="1"/>
     <row r="31" ht="15" customHeight="1"/>
@@ -8749,8 +9517,6 @@
     <row r="38" ht="15" customHeight="1"/>
     <row r="39" ht="15" customHeight="1"/>
     <row r="40" ht="15" customHeight="1"/>
-    <row r="41" ht="15" customHeight="1"/>
-    <row r="42" ht="15" customHeight="1"/>
     <row r="43" ht="15" customHeight="1"/>
     <row r="44" ht="15" customHeight="1"/>
     <row r="45" ht="15" customHeight="1"/>
@@ -8759,768 +9525,1706 @@
     <row r="48" ht="15" customHeight="1"/>
     <row r="49" ht="15" customHeight="1"/>
     <row r="50" ht="15" customHeight="1"/>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="51" ht="15" customHeight="1"/>
+    <row r="52" ht="15" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="15" customHeight="1"/>
+    <row r="55" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="15" customHeight="1"/>
+    <row r="59" ht="15" customHeight="1"/>
+    <row r="60" ht="15" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="15" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1"/>
+    <row r="67" ht="15" customHeight="1"/>
+    <row r="68" ht="15" customHeight="1"/>
+    <row r="69" ht="15" customHeight="1"/>
+    <row r="70" ht="15" customHeight="1"/>
+    <row r="71" ht="15" customHeight="1"/>
+    <row r="72" ht="15" customHeight="1"/>
+    <row r="73" ht="15" customHeight="1"/>
+    <row r="74" ht="15" customHeight="1"/>
+    <row r="75" ht="15" customHeight="1"/>
+    <row r="76" ht="15" customHeight="1"/>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="78" ht="15" customHeight="1"/>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>Curve data (mean of 3 folds)</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="48.5" customHeight="1">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="82" ht="75.5" customHeight="1">
+      <c r="A82" s="5" t="inlineStr">
         <is>
           <t>Epoch</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B82" s="5" t="inlineStr">
         <is>
           <t>Early Fusion + CE: train SeK</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C82" s="5" t="inlineStr">
         <is>
           <t>Early Fusion + CE: val SeK</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D82" s="5" t="inlineStr">
         <is>
           <t>SSCD + CE: train SeK</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E82" s="5" t="inlineStr">
         <is>
           <t>SSCD + CE: val SeK</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F82" s="5" t="inlineStr">
         <is>
           <t>BiSR + CE: train SeK</t>
         </is>
       </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="G82" s="5" t="inlineStr">
         <is>
           <t>BiSR + CE: val SeK</t>
         </is>
       </c>
-      <c r="H54" s="5" t="inlineStr">
+      <c r="H82" s="5" t="inlineStr">
         <is>
           <t>BiSR + WCE + Dice: train SeK</t>
         </is>
       </c>
-      <c r="I54" s="5" t="inlineStr">
+      <c r="I82" s="5" t="inlineStr">
         <is>
           <t>BiSR + WCE + Dice: val SeK</t>
         </is>
       </c>
-      <c r="J54" s="5" t="inlineStr">
+      <c r="J82" s="5" t="inlineStr">
         <is>
           <t>BiSR + CE + Dice: train SeK</t>
         </is>
       </c>
-      <c r="K54" s="5" t="inlineStr">
+      <c r="K82" s="5" t="inlineStr">
         <is>
           <t>BiSR + CE + Dice: val SeK</t>
         </is>
       </c>
-    </row>
-    <row r="55" ht="18.5" customHeight="1">
-      <c r="A55" s="56" t="n">
+      <c r="L82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Weighted CE: train SeK</t>
+        </is>
+      </c>
+      <c r="M82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Weighted CE: val SeK</t>
+        </is>
+      </c>
+      <c r="N82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Median-freq: train SeK</t>
+        </is>
+      </c>
+      <c r="O82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Median-freq: val SeK</t>
+        </is>
+      </c>
+      <c r="P82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Class-balanced: train SeK</t>
+        </is>
+      </c>
+      <c r="Q82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Class-balanced: val SeK</t>
+        </is>
+      </c>
+      <c r="R82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Focal: train SeK</t>
+        </is>
+      </c>
+      <c r="S82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + Focal: val SeK</t>
+        </is>
+      </c>
+      <c r="T82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + CE + rare sampling: train SeK</t>
+        </is>
+      </c>
+      <c r="U82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + CE + rare sampling: val SeK</t>
+        </is>
+      </c>
+      <c r="V82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + WCE + Dice + rare sampling: train SeK</t>
+        </is>
+      </c>
+      <c r="W82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + WCE + Dice + rare sampling: val SeK</t>
+        </is>
+      </c>
+      <c r="X82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + OHEM: train SeK</t>
+        </is>
+      </c>
+      <c r="Y82" s="5" t="inlineStr">
+        <is>
+          <t>BiSR + OHEM: val SeK</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18.5" customHeight="1">
+      <c r="A83" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="B55" s="37" t="n">
+      <c r="B83" s="37" t="n">
         <v>-8.019840239144273</v>
       </c>
-      <c r="C55" s="37" t="n">
+      <c r="C83" s="37" t="n">
         <v>-9.085370840449466</v>
       </c>
-      <c r="D55" s="37" t="n">
+      <c r="D83" s="37" t="n">
         <v>1.517827638620062</v>
       </c>
-      <c r="E55" s="37" t="n">
+      <c r="E83" s="37" t="n">
         <v>0.3404761560565535</v>
       </c>
-      <c r="F55" s="37" t="n">
+      <c r="F83" s="37" t="n">
         <v>1.679210469154502</v>
       </c>
-      <c r="G55" s="37" t="n">
+      <c r="G83" s="37" t="n">
         <v>0.5091279017640838</v>
       </c>
-      <c r="H55" s="37" t="n">
+      <c r="H83" s="37" t="n">
         <v>4.44134593855201</v>
       </c>
-      <c r="I55" s="37" t="n">
+      <c r="I83" s="37" t="n">
         <v>3.279226070962359</v>
       </c>
-      <c r="J55" s="37" t="n">
+      <c r="J83" s="37" t="n">
         <v>3.663539539420352</v>
       </c>
-      <c r="K55" s="37" t="n">
+      <c r="K83" s="37" t="n">
         <v>2.496566762510674</v>
       </c>
-    </row>
-    <row r="56" ht="18.5" customHeight="1">
-      <c r="A56" s="57" t="n">
+      <c r="L83" s="37" t="n">
+        <v>3.009504844071606</v>
+      </c>
+      <c r="M83" s="37" t="n">
+        <v>1.894016891190606</v>
+      </c>
+      <c r="N83" s="37" t="n">
+        <v>2.093545987406457</v>
+      </c>
+      <c r="O83" s="37" t="n">
+        <v>1.081184740848382</v>
+      </c>
+      <c r="P83" s="37" t="n">
+        <v>2.741539369128389</v>
+      </c>
+      <c r="Q83" s="37" t="n">
+        <v>1.681726452811396</v>
+      </c>
+      <c r="R83" s="37" t="n">
+        <v>2.70283009178323</v>
+      </c>
+      <c r="S83" s="37" t="n">
+        <v>1.669930201360692</v>
+      </c>
+      <c r="T83" s="37" t="n">
+        <v>1.330104833887798</v>
+      </c>
+      <c r="U83" s="37" t="n">
+        <v>0.01891248695492041</v>
+      </c>
+      <c r="V83" s="37" t="n">
+        <v>3.865580347856438</v>
+      </c>
+      <c r="W83" s="37" t="n">
+        <v>2.666978621627395</v>
+      </c>
+      <c r="X83" s="37" t="n">
+        <v>-5.06655230683639</v>
+      </c>
+      <c r="Y83" s="37" t="n">
+        <v>-5.326042542949577</v>
+      </c>
+    </row>
+    <row r="84" ht="18.5" customHeight="1">
+      <c r="A84" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="B56" s="41" t="n">
+      <c r="B84" s="41" t="n">
         <v>-1.728705110584415</v>
       </c>
-      <c r="C56" s="41" t="n">
+      <c r="C84" s="41" t="n">
         <v>-2.308614301747373</v>
       </c>
-      <c r="D56" s="41" t="n">
+      <c r="D84" s="41" t="n">
         <v>8.899115317867087</v>
       </c>
-      <c r="E56" s="41" t="n">
+      <c r="E84" s="41" t="n">
         <v>7.505325813176337</v>
       </c>
-      <c r="F56" s="41" t="n">
+      <c r="F84" s="41" t="n">
         <v>8.787635643683368</v>
       </c>
-      <c r="G56" s="41" t="n">
+      <c r="G84" s="41" t="n">
         <v>7.47298305920918</v>
       </c>
-      <c r="H56" s="41" t="n">
+      <c r="H84" s="41" t="n">
         <v>10.16731398364418</v>
       </c>
-      <c r="I56" s="41" t="n">
+      <c r="I84" s="41" t="n">
         <v>8.521336194144901</v>
       </c>
-      <c r="J56" s="41" t="n">
+      <c r="J84" s="41" t="n">
         <v>10.35872525368809</v>
       </c>
-      <c r="K56" s="41" t="n">
+      <c r="K84" s="41" t="n">
         <v>8.604658241885325</v>
       </c>
-    </row>
-    <row r="57" ht="18.5" customHeight="1">
-      <c r="A57" s="56" t="n">
+      <c r="L84" s="41" t="n">
+        <v>9.909933198618734</v>
+      </c>
+      <c r="M84" s="41" t="n">
+        <v>8.292545366158173</v>
+      </c>
+      <c r="N84" s="41" t="n">
+        <v>8.461136562305226</v>
+      </c>
+      <c r="O84" s="41" t="n">
+        <v>7.028336044173812</v>
+      </c>
+      <c r="P84" s="41" t="n">
+        <v>9.262690681645561</v>
+      </c>
+      <c r="Q84" s="41" t="n">
+        <v>7.752189735344465</v>
+      </c>
+      <c r="R84" s="41" t="n">
+        <v>8.843288217620028</v>
+      </c>
+      <c r="S84" s="41" t="n">
+        <v>6.890133769057048</v>
+      </c>
+      <c r="T84" s="41" t="n">
+        <v>8.875751306394406</v>
+      </c>
+      <c r="U84" s="41" t="n">
+        <v>6.934759234703932</v>
+      </c>
+      <c r="V84" s="41" t="n">
+        <v>10.07859784090252</v>
+      </c>
+      <c r="W84" s="41" t="n">
+        <v>7.691398904818864</v>
+      </c>
+      <c r="X84" s="41" t="n">
+        <v>-3.912124505688055</v>
+      </c>
+      <c r="Y84" s="41" t="n">
+        <v>-4.814937005148878</v>
+      </c>
+    </row>
+    <row r="85" ht="18.5" customHeight="1">
+      <c r="A85" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="B57" s="37" t="n">
+      <c r="B85" s="37" t="n">
         <v>0.4008647300068447</v>
       </c>
-      <c r="C57" s="37" t="n">
+      <c r="C85" s="37" t="n">
         <v>-0.2231251534836043</v>
       </c>
-      <c r="D57" s="37" t="n">
+      <c r="D85" s="37" t="n">
         <v>10.82209966906606</v>
       </c>
-      <c r="E57" s="37" t="n">
+      <c r="E85" s="37" t="n">
         <v>9.178044773102512</v>
       </c>
-      <c r="F57" s="37" t="n">
+      <c r="F85" s="37" t="n">
         <v>10.8633429948913</v>
       </c>
-      <c r="G57" s="37" t="n">
+      <c r="G85" s="37" t="n">
         <v>9.279337299389281</v>
       </c>
-      <c r="H57" s="37" t="n">
+      <c r="H85" s="37" t="n">
         <v>12.13407827999307</v>
       </c>
-      <c r="I57" s="37" t="n">
+      <c r="I85" s="37" t="n">
         <v>10.09401234510733</v>
       </c>
-      <c r="J57" s="37" t="n">
+      <c r="J85" s="37" t="n">
         <v>12.24615907273666</v>
       </c>
-      <c r="K57" s="37" t="n">
+      <c r="K85" s="37" t="n">
         <v>10.12363645934475</v>
       </c>
-    </row>
-    <row r="58" ht="18.5" customHeight="1">
-      <c r="A58" s="57" t="n">
+      <c r="L85" s="37" t="n">
+        <v>12.23218009838717</v>
+      </c>
+      <c r="M85" s="37" t="n">
+        <v>10.18548440290681</v>
+      </c>
+      <c r="N85" s="37" t="n">
+        <v>10.5481967640611</v>
+      </c>
+      <c r="O85" s="37" t="n">
+        <v>8.71693681107431</v>
+      </c>
+      <c r="P85" s="37" t="n">
+        <v>11.47302941445717</v>
+      </c>
+      <c r="Q85" s="37" t="n">
+        <v>9.62138250616127</v>
+      </c>
+      <c r="R85" s="37" t="n">
+        <v>10.68072062766441</v>
+      </c>
+      <c r="S85" s="37" t="n">
+        <v>8.649401380924569</v>
+      </c>
+      <c r="T85" s="37" t="n">
+        <v>11.30955253967828</v>
+      </c>
+      <c r="U85" s="37" t="n">
+        <v>8.969867166530436</v>
+      </c>
+      <c r="V85" s="37" t="n">
+        <v>12.29033491107394</v>
+      </c>
+      <c r="W85" s="37" t="n">
+        <v>9.663251685297725</v>
+      </c>
+      <c r="X85" s="37" t="n">
+        <v>-2.224997033598683</v>
+      </c>
+      <c r="Y85" s="37" t="n">
+        <v>-3.176067324288626</v>
+      </c>
+    </row>
+    <row r="86" ht="18.5" customHeight="1">
+      <c r="A86" s="57" t="n">
         <v>4</v>
       </c>
-      <c r="B58" s="41" t="n">
+      <c r="B86" s="41" t="n">
         <v>2.279009815627986</v>
       </c>
-      <c r="C58" s="41" t="n">
+      <c r="C86" s="41" t="n">
         <v>1.189929223446843</v>
       </c>
-      <c r="D58" s="41" t="n">
+      <c r="D86" s="41" t="n">
         <v>13.4351724372879</v>
       </c>
-      <c r="E58" s="41" t="n">
+      <c r="E86" s="41" t="n">
         <v>10.6064350479089</v>
       </c>
-      <c r="F58" s="41" t="n">
+      <c r="F86" s="41" t="n">
         <v>13.22946005157054</v>
       </c>
-      <c r="G58" s="41" t="n">
+      <c r="G86" s="41" t="n">
         <v>10.46293655648843</v>
       </c>
-      <c r="H58" s="41" t="n">
+      <c r="H86" s="41" t="n">
         <v>14.48294567590852</v>
       </c>
-      <c r="I58" s="41" t="n">
+      <c r="I86" s="41" t="n">
         <v>11.56199244154197</v>
       </c>
-      <c r="J58" s="41" t="n">
+      <c r="J86" s="41" t="n">
         <v>14.26211263917511</v>
       </c>
-      <c r="K58" s="41" t="n">
+      <c r="K86" s="41" t="n">
         <v>11.50817314331024</v>
       </c>
-    </row>
-    <row r="59" ht="18.5" customHeight="1">
-      <c r="A59" s="56" t="n">
+      <c r="L86" s="41" t="n">
+        <v>14.01085824679374</v>
+      </c>
+      <c r="M86" s="41" t="n">
+        <v>11.31206537602668</v>
+      </c>
+      <c r="N86" s="41" t="n">
+        <v>13.09331497466297</v>
+      </c>
+      <c r="O86" s="41" t="n">
+        <v>10.65088502318131</v>
+      </c>
+      <c r="P86" s="41" t="n">
+        <v>13.59971649352259</v>
+      </c>
+      <c r="Q86" s="41" t="n">
+        <v>11.04977427877669</v>
+      </c>
+      <c r="R86" s="41" t="n">
+        <v>12.34532198143083</v>
+      </c>
+      <c r="S86" s="41" t="n">
+        <v>9.891293266877485</v>
+      </c>
+      <c r="T86" s="41" t="n">
+        <v>13.75746317928693</v>
+      </c>
+      <c r="U86" s="41" t="n">
+        <v>10.82221042186662</v>
+      </c>
+      <c r="V86" s="41" t="n">
+        <v>13.98754893901647</v>
+      </c>
+      <c r="W86" s="41" t="n">
+        <v>10.99348794219114</v>
+      </c>
+      <c r="X86" s="41" t="n">
+        <v>0.1312222820685586</v>
+      </c>
+      <c r="Y86" s="41" t="n">
+        <v>-0.9972430447330449</v>
+      </c>
+    </row>
+    <row r="87" ht="18.5" customHeight="1">
+      <c r="A87" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="B59" s="37" t="n">
+      <c r="B87" s="37" t="n">
         <v>3.912007822148761</v>
       </c>
-      <c r="C59" s="37" t="n">
+      <c r="C87" s="37" t="n">
         <v>2.55416489125884</v>
       </c>
-      <c r="D59" s="37" t="n">
+      <c r="D87" s="37" t="n">
         <v>14.95524091912318</v>
       </c>
-      <c r="E59" s="37" t="n">
+      <c r="E87" s="37" t="n">
         <v>11.21768758551962</v>
       </c>
-      <c r="F59" s="37" t="n">
+      <c r="F87" s="37" t="n">
         <v>14.47301814222977</v>
       </c>
-      <c r="G59" s="37" t="n">
+      <c r="G87" s="37" t="n">
         <v>11.22846024508185</v>
       </c>
-      <c r="H59" s="37" t="n">
+      <c r="H87" s="37" t="n">
         <v>15.12790666015765</v>
       </c>
-      <c r="I59" s="37" t="n">
+      <c r="I87" s="37" t="n">
         <v>11.89674113751082</v>
       </c>
-      <c r="J59" s="37" t="n">
+      <c r="J87" s="37" t="n">
         <v>15.25865622339026</v>
       </c>
-      <c r="K59" s="37" t="n">
+      <c r="K87" s="37" t="n">
         <v>11.68198339759578</v>
       </c>
-    </row>
-    <row r="60" ht="18.5" customHeight="1">
-      <c r="A60" s="57" t="n">
+      <c r="L87" s="37" t="n">
+        <v>14.89080177865355</v>
+      </c>
+      <c r="M87" s="37" t="n">
+        <v>11.81583529104268</v>
+      </c>
+      <c r="N87" s="37" t="n">
+        <v>13.25340010710389</v>
+      </c>
+      <c r="O87" s="37" t="n">
+        <v>10.50356458161344</v>
+      </c>
+      <c r="P87" s="37" t="n">
+        <v>13.91107019962171</v>
+      </c>
+      <c r="Q87" s="37" t="n">
+        <v>11.21694498062192</v>
+      </c>
+      <c r="R87" s="37" t="n">
+        <v>12.82217538430554</v>
+      </c>
+      <c r="S87" s="37" t="n">
+        <v>10.21297098247231</v>
+      </c>
+      <c r="T87" s="37" t="n">
+        <v>13.50586459979794</v>
+      </c>
+      <c r="U87" s="37" t="n">
+        <v>10.18848221544003</v>
+      </c>
+      <c r="V87" s="37" t="n">
+        <v>14.15985386671594</v>
+      </c>
+      <c r="W87" s="37" t="n">
+        <v>11.24230848280891</v>
+      </c>
+      <c r="X87" s="37" t="n">
+        <v>-0.6181986705133506</v>
+      </c>
+      <c r="Y87" s="37" t="n">
+        <v>-1.000160197254512</v>
+      </c>
+    </row>
+    <row r="88" ht="18.5" customHeight="1">
+      <c r="A88" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="B60" s="41" t="n">
+      <c r="B88" s="41" t="n">
         <v>3.253362987115743</v>
       </c>
-      <c r="C60" s="41" t="n">
+      <c r="C88" s="41" t="n">
         <v>2.024629800034</v>
       </c>
-      <c r="D60" s="41" t="n">
+      <c r="D88" s="41" t="n">
         <v>14.61336533390383</v>
       </c>
-      <c r="E60" s="41" t="n">
+      <c r="E88" s="41" t="n">
         <v>11.04708836626668</v>
       </c>
-      <c r="F60" s="41" t="n">
+      <c r="F88" s="41" t="n">
         <v>14.23669108299754</v>
       </c>
-      <c r="G60" s="41" t="n">
+      <c r="G88" s="41" t="n">
         <v>11.08234189337929</v>
       </c>
-      <c r="H60" s="41" t="n">
+      <c r="H88" s="41" t="n">
         <v>16.01857037541095</v>
       </c>
-      <c r="I60" s="41" t="n">
+      <c r="I88" s="41" t="n">
         <v>12.35535376157269</v>
       </c>
-      <c r="J60" s="41" t="n">
+      <c r="J88" s="41" t="n">
         <v>15.98968187459353</v>
       </c>
-      <c r="K60" s="41" t="n">
+      <c r="K88" s="41" t="n">
         <v>12.28056554470235</v>
       </c>
-    </row>
-    <row r="61" ht="18.5" customHeight="1">
-      <c r="A61" s="56" t="n">
+      <c r="L88" s="41" t="n">
+        <v>15.56066339332285</v>
+      </c>
+      <c r="M88" s="41" t="n">
+        <v>12.03295274514173</v>
+      </c>
+      <c r="N88" s="41" t="n">
+        <v>14.37836910426911</v>
+      </c>
+      <c r="O88" s="41" t="n">
+        <v>11.24224963226931</v>
+      </c>
+      <c r="P88" s="41" t="n">
+        <v>15.19941585459873</v>
+      </c>
+      <c r="Q88" s="41" t="n">
+        <v>11.897702215046</v>
+      </c>
+      <c r="R88" s="41" t="n">
+        <v>14.36015820083191</v>
+      </c>
+      <c r="S88" s="41" t="n">
+        <v>11.34507392352159</v>
+      </c>
+      <c r="T88" s="41" t="n">
+        <v>15.5573726574795</v>
+      </c>
+      <c r="U88" s="41" t="n">
+        <v>11.92991999807233</v>
+      </c>
+      <c r="V88" s="41" t="n">
+        <v>15.4298002375434</v>
+      </c>
+      <c r="W88" s="41" t="n">
+        <v>12.20955184721342</v>
+      </c>
+      <c r="X88" s="41" t="n">
+        <v>1.360042264019443</v>
+      </c>
+      <c r="Y88" s="41" t="n">
+        <v>0.595693924178592</v>
+      </c>
+    </row>
+    <row r="89" ht="18.5" customHeight="1">
+      <c r="A89" s="56" t="n">
         <v>7</v>
       </c>
-      <c r="B61" s="37" t="n">
+      <c r="B89" s="37" t="n">
         <v>5.276670246388964</v>
       </c>
-      <c r="C61" s="37" t="n">
+      <c r="C89" s="37" t="n">
         <v>3.486571840591929</v>
       </c>
-      <c r="D61" s="37" t="n">
+      <c r="D89" s="37" t="n">
         <v>16.97421905170832</v>
       </c>
-      <c r="E61" s="37" t="n">
+      <c r="E89" s="37" t="n">
         <v>12.45104609202909</v>
       </c>
-      <c r="F61" s="37" t="n">
+      <c r="F89" s="37" t="n">
         <v>16.56903412845136</v>
       </c>
-      <c r="G61" s="37" t="n">
+      <c r="G89" s="37" t="n">
         <v>12.54320558492488</v>
       </c>
-      <c r="H61" s="37" t="n">
+      <c r="H89" s="37" t="n">
         <v>16.41983337540134</v>
       </c>
-      <c r="I61" s="37" t="n">
+      <c r="I89" s="37" t="n">
         <v>12.6852009600241</v>
       </c>
-      <c r="J61" s="37" t="n">
+      <c r="J89" s="37" t="n">
         <v>17.13032899201437</v>
       </c>
-      <c r="K61" s="37" t="n">
+      <c r="K89" s="37" t="n">
         <v>12.88996672130515</v>
       </c>
-    </row>
-    <row r="62" ht="18.5" customHeight="1">
-      <c r="A62" s="57" t="n">
+      <c r="L89" s="37" t="n">
+        <v>15.86523444864903</v>
+      </c>
+      <c r="M89" s="37" t="n">
+        <v>12.42628411876575</v>
+      </c>
+      <c r="N89" s="37" t="n">
+        <v>15.38509366753923</v>
+      </c>
+      <c r="O89" s="37" t="n">
+        <v>12.00722496747445</v>
+      </c>
+      <c r="P89" s="37" t="n">
+        <v>15.71730855574356</v>
+      </c>
+      <c r="Q89" s="37" t="n">
+        <v>12.23652532374136</v>
+      </c>
+      <c r="R89" s="37" t="n">
+        <v>14.15491133999654</v>
+      </c>
+      <c r="S89" s="37" t="n">
+        <v>11.35471043411968</v>
+      </c>
+      <c r="T89" s="37" t="n">
+        <v>15.82261755641343</v>
+      </c>
+      <c r="U89" s="37" t="n">
+        <v>11.76803546338359</v>
+      </c>
+      <c r="V89" s="37" t="n">
+        <v>16.5452961290881</v>
+      </c>
+      <c r="W89" s="37" t="n">
+        <v>12.37391612832058</v>
+      </c>
+      <c r="X89" s="37" t="n">
+        <v>-1.036388779872201</v>
+      </c>
+      <c r="Y89" s="37" t="n">
+        <v>-1.538250779137525</v>
+      </c>
+    </row>
+    <row r="90" ht="18.5" customHeight="1">
+      <c r="A90" s="57" t="n">
         <v>8</v>
       </c>
-      <c r="B62" s="41" t="n">
+      <c r="B90" s="41" t="n">
         <v>7.360769791737428</v>
       </c>
-      <c r="C62" s="41" t="n">
+      <c r="C90" s="41" t="n">
         <v>4.817640508738741</v>
       </c>
-      <c r="D62" s="41" t="n">
+      <c r="D90" s="41" t="n">
         <v>18.14453747262751</v>
       </c>
-      <c r="E62" s="41" t="n">
+      <c r="E90" s="41" t="n">
         <v>12.45986127269612</v>
       </c>
-      <c r="F62" s="41" t="n">
+      <c r="F90" s="41" t="n">
         <v>17.58264283040106</v>
       </c>
-      <c r="G62" s="41" t="n">
+      <c r="G90" s="41" t="n">
         <v>12.74055804541727</v>
       </c>
-      <c r="H62" s="41" t="n">
+      <c r="H90" s="41" t="n">
         <v>18.14657239102235</v>
       </c>
-      <c r="I62" s="41" t="n">
+      <c r="I90" s="41" t="n">
         <v>13.47185013979055</v>
       </c>
-      <c r="J62" s="41" t="n">
+      <c r="J90" s="41" t="n">
         <v>18.53202329067662</v>
       </c>
-      <c r="K62" s="41" t="n">
+      <c r="K90" s="41" t="n">
         <v>13.462550269514</v>
       </c>
-    </row>
-    <row r="63" ht="18.5" customHeight="1">
-      <c r="A63" s="56" t="n">
+      <c r="L90" s="41" t="n">
+        <v>17.5671716623861</v>
+      </c>
+      <c r="M90" s="41" t="n">
+        <v>13.17710729462781</v>
+      </c>
+      <c r="N90" s="41" t="n">
+        <v>16.20550162798401</v>
+      </c>
+      <c r="O90" s="41" t="n">
+        <v>12.40224845863492</v>
+      </c>
+      <c r="P90" s="41" t="n">
+        <v>16.9517612827499</v>
+      </c>
+      <c r="Q90" s="41" t="n">
+        <v>12.86090038171586</v>
+      </c>
+      <c r="R90" s="41" t="n">
+        <v>15.57444341897996</v>
+      </c>
+      <c r="S90" s="41" t="n">
+        <v>11.92801696882318</v>
+      </c>
+      <c r="T90" s="41" t="n">
+        <v>16.48778473457368</v>
+      </c>
+      <c r="U90" s="41" t="n">
+        <v>12.26814586503762</v>
+      </c>
+      <c r="V90" s="41" t="n">
+        <v>16.97230628708276</v>
+      </c>
+      <c r="W90" s="41" t="n">
+        <v>12.71375749601872</v>
+      </c>
+      <c r="X90" s="41" t="n">
+        <v>0.6915892687100169</v>
+      </c>
+      <c r="Y90" s="41" t="n">
+        <v>-0.05342157690203594</v>
+      </c>
+    </row>
+    <row r="91" ht="18.5" customHeight="1">
+      <c r="A91" s="56" t="n">
         <v>9</v>
       </c>
-      <c r="B63" s="37" t="n">
+      <c r="B91" s="37" t="n">
         <v>7.098795720390233</v>
       </c>
-      <c r="C63" s="37" t="n">
+      <c r="C91" s="37" t="n">
         <v>4.802987497216051</v>
       </c>
-      <c r="D63" s="37" t="n">
+      <c r="D91" s="37" t="n">
         <v>18.47348931532116</v>
       </c>
-      <c r="E63" s="37" t="n">
+      <c r="E91" s="37" t="n">
         <v>12.53284583958772</v>
       </c>
-      <c r="F63" s="37" t="n">
+      <c r="F91" s="37" t="n">
         <v>17.85968261184047</v>
       </c>
-      <c r="G63" s="37" t="n">
+      <c r="G91" s="37" t="n">
         <v>12.93319365708107</v>
       </c>
-      <c r="H63" s="37" t="n">
+      <c r="H91" s="37" t="n">
         <v>18.84060323491924</v>
       </c>
-      <c r="I63" s="37" t="n">
+      <c r="I91" s="37" t="n">
         <v>13.63630061565906</v>
       </c>
-      <c r="J63" s="37" t="n">
+      <c r="J91" s="37" t="n">
         <v>19.51969362535073</v>
       </c>
-      <c r="K63" s="37" t="n">
+      <c r="K91" s="37" t="n">
         <v>13.80506322532518</v>
       </c>
-    </row>
-    <row r="64" ht="18.5" customHeight="1">
-      <c r="A64" s="57" t="n">
+      <c r="L91" s="37" t="n">
+        <v>18.66816367474186</v>
+      </c>
+      <c r="M91" s="37" t="n">
+        <v>13.48799839272867</v>
+      </c>
+      <c r="N91" s="37" t="n">
+        <v>16.59685542191176</v>
+      </c>
+      <c r="O91" s="37" t="n">
+        <v>12.69236822778012</v>
+      </c>
+      <c r="P91" s="37" t="n">
+        <v>17.52923216435777</v>
+      </c>
+      <c r="Q91" s="37" t="n">
+        <v>13.1491934528433</v>
+      </c>
+      <c r="R91" s="37" t="n">
+        <v>16.58664425890168</v>
+      </c>
+      <c r="S91" s="37" t="n">
+        <v>12.34496367325668</v>
+      </c>
+      <c r="T91" s="37" t="n">
+        <v>17.35562518446126</v>
+      </c>
+      <c r="U91" s="37" t="n">
+        <v>12.64149390477939</v>
+      </c>
+      <c r="V91" s="37" t="n">
+        <v>17.84360264258356</v>
+      </c>
+      <c r="W91" s="37" t="n">
+        <v>13.22307716532633</v>
+      </c>
+      <c r="X91" s="37" t="n">
+        <v>1.85118697842957</v>
+      </c>
+      <c r="Y91" s="37" t="n">
+        <v>1.164116320070683</v>
+      </c>
+    </row>
+    <row r="92" ht="18.5" customHeight="1">
+      <c r="A92" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="B64" s="41" t="n">
+      <c r="B92" s="41" t="n">
         <v>6.71424172650577</v>
       </c>
-      <c r="C64" s="41" t="n">
+      <c r="C92" s="41" t="n">
         <v>4.318353073003482</v>
       </c>
-      <c r="D64" s="41" t="n">
+      <c r="D92" s="41" t="n">
         <v>18.50246395246403</v>
       </c>
-      <c r="E64" s="41" t="n">
+      <c r="E92" s="41" t="n">
         <v>11.9197870056203</v>
       </c>
-      <c r="F64" s="41" t="n">
+      <c r="F92" s="41" t="n">
         <v>18.20768329655014</v>
       </c>
-      <c r="G64" s="41" t="n">
+      <c r="G92" s="41" t="n">
         <v>12.85181884128474</v>
       </c>
-      <c r="H64" s="41" t="n">
+      <c r="H92" s="41" t="n">
         <v>19.6652966807824</v>
       </c>
-      <c r="I64" s="41" t="n">
+      <c r="I92" s="41" t="n">
         <v>13.87750527783653</v>
       </c>
-      <c r="J64" s="41" t="n">
+      <c r="J92" s="41" t="n">
         <v>20.01822289110888</v>
       </c>
-      <c r="K64" s="41" t="n">
+      <c r="K92" s="41" t="n">
         <v>13.9365255094347</v>
       </c>
-    </row>
-    <row r="65" ht="18.5" customHeight="1">
-      <c r="A65" s="56" t="n">
+      <c r="L92" s="41" t="n">
+        <v>19.28373312277044</v>
+      </c>
+      <c r="M92" s="41" t="n">
+        <v>13.59787972649484</v>
+      </c>
+      <c r="N92" s="41" t="n">
+        <v>17.28000891519635</v>
+      </c>
+      <c r="O92" s="41" t="n">
+        <v>12.9373336254783</v>
+      </c>
+      <c r="P92" s="41" t="n">
+        <v>18.01180216059547</v>
+      </c>
+      <c r="Q92" s="41" t="n">
+        <v>13.29180996916003</v>
+      </c>
+      <c r="R92" s="41" t="n">
+        <v>16.80904887451198</v>
+      </c>
+      <c r="S92" s="41" t="n">
+        <v>12.50356038060262</v>
+      </c>
+      <c r="T92" s="41" t="n">
+        <v>17.11817752857672</v>
+      </c>
+      <c r="U92" s="41" t="n">
+        <v>11.79762461470285</v>
+      </c>
+      <c r="V92" s="41" t="n">
+        <v>18.43406716138331</v>
+      </c>
+      <c r="W92" s="41" t="n">
+        <v>12.98891858939958</v>
+      </c>
+      <c r="X92" s="41" t="n">
+        <v>-1.500991471411738</v>
+      </c>
+      <c r="Y92" s="41" t="n">
+        <v>-1.910024481820946</v>
+      </c>
+    </row>
+    <row r="93" ht="18.5" customHeight="1">
+      <c r="A93" s="56" t="n">
         <v>11</v>
       </c>
-      <c r="B65" s="37" t="n">
+      <c r="B93" s="37" t="n">
         <v>7.604426146870488</v>
       </c>
-      <c r="C65" s="37" t="n">
+      <c r="C93" s="37" t="n">
         <v>4.795897153888503</v>
       </c>
-      <c r="D65" s="37" t="n">
+      <c r="D93" s="37" t="n">
         <v>19.44774030193662</v>
       </c>
-      <c r="E65" s="37" t="n">
+      <c r="E93" s="37" t="n">
         <v>11.98753031061223</v>
       </c>
-      <c r="F65" s="37" t="n">
+      <c r="F93" s="37" t="n">
         <v>18.784590296776</v>
       </c>
-      <c r="G65" s="37" t="n">
+      <c r="G93" s="37" t="n">
         <v>12.76155603998925</v>
       </c>
-      <c r="H65" s="37" t="n">
+      <c r="H93" s="37" t="n">
         <v>20.20343912627485</v>
       </c>
-      <c r="I65" s="37" t="n">
+      <c r="I93" s="37" t="n">
         <v>13.85485691061338</v>
       </c>
-      <c r="J65" s="37" t="n">
+      <c r="J93" s="37" t="n">
         <v>20.1648888686858</v>
       </c>
-      <c r="K65" s="37" t="n">
+      <c r="K93" s="37" t="n">
         <v>13.63480513830139</v>
       </c>
-    </row>
-    <row r="66" ht="18.5" customHeight="1">
-      <c r="A66" s="57" t="n">
+      <c r="L93" s="37" t="n">
+        <v>19.37136724628565</v>
+      </c>
+      <c r="M93" s="37" t="n">
+        <v>13.73300870878879</v>
+      </c>
+      <c r="N93" s="37" t="n">
+        <v>17.34380569558573</v>
+      </c>
+      <c r="O93" s="37" t="n">
+        <v>12.736388055792</v>
+      </c>
+      <c r="P93" s="37" t="n">
+        <v>18.49282160711517</v>
+      </c>
+      <c r="Q93" s="37" t="n">
+        <v>13.34854933526784</v>
+      </c>
+      <c r="R93" s="37" t="n">
+        <v>17.49024717001804</v>
+      </c>
+      <c r="S93" s="37" t="n">
+        <v>12.57489264890189</v>
+      </c>
+      <c r="T93" s="37" t="n">
+        <v>18.96091997734181</v>
+      </c>
+      <c r="U93" s="37" t="n">
+        <v>13.08172950879008</v>
+      </c>
+      <c r="V93" s="37" t="n">
+        <v>18.89100064186167</v>
+      </c>
+      <c r="W93" s="37" t="n">
+        <v>13.20682197657883</v>
+      </c>
+      <c r="X93" s="37" t="n">
+        <v>1.951782900297982</v>
+      </c>
+      <c r="Y93" s="37" t="n">
+        <v>0.8176032936923812</v>
+      </c>
+    </row>
+    <row r="94" ht="18.5" customHeight="1">
+      <c r="A94" s="57" t="n">
         <v>12</v>
       </c>
-      <c r="B66" s="41" t="n">
+      <c r="B94" s="41" t="n">
         <v>9.410837865592235</v>
       </c>
-      <c r="C66" s="41" t="n">
+      <c r="C94" s="41" t="n">
         <v>6.198327681569695</v>
       </c>
-      <c r="D66" s="41" t="n">
+      <c r="D94" s="41" t="n">
         <v>21.50849030212062</v>
       </c>
-      <c r="E66" s="41" t="n">
+      <c r="E94" s="41" t="n">
         <v>12.95088227552498</v>
       </c>
-      <c r="F66" s="41" t="n">
+      <c r="F94" s="41" t="n">
         <v>20.3957221813331</v>
       </c>
-      <c r="G66" s="41" t="n">
+      <c r="G94" s="41" t="n">
         <v>13.59036202890574</v>
       </c>
-      <c r="H66" s="41" t="n">
+      <c r="H94" s="41" t="n">
         <v>21.07086340154639</v>
       </c>
-      <c r="I66" s="41" t="n">
+      <c r="I94" s="41" t="n">
         <v>14.27196536844385</v>
       </c>
-      <c r="J66" s="41" t="n">
+      <c r="J94" s="41" t="n">
         <v>21.45303910319052</v>
       </c>
-      <c r="K66" s="41" t="n">
+      <c r="K94" s="41" t="n">
         <v>14.3556347828075</v>
       </c>
-    </row>
-    <row r="67" ht="18.5" customHeight="1">
-      <c r="A67" s="56" t="n">
+      <c r="L94" s="41" t="n">
+        <v>20.48142157275731</v>
+      </c>
+      <c r="M94" s="41" t="n">
+        <v>14.17989798492608</v>
+      </c>
+      <c r="N94" s="41" t="n">
+        <v>18.372718374592</v>
+      </c>
+      <c r="O94" s="41" t="n">
+        <v>13.56644668106112</v>
+      </c>
+      <c r="P94" s="41" t="n">
+        <v>19.52035841052173</v>
+      </c>
+      <c r="Q94" s="41" t="n">
+        <v>14.07165917981957</v>
+      </c>
+      <c r="R94" s="41" t="n">
+        <v>17.93134637878278</v>
+      </c>
+      <c r="S94" s="41" t="n">
+        <v>13.011217631178</v>
+      </c>
+      <c r="T94" s="41" t="n">
+        <v>19.20782799039052</v>
+      </c>
+      <c r="U94" s="41" t="n">
+        <v>13.02839530241062</v>
+      </c>
+      <c r="V94" s="41" t="n">
+        <v>19.91745681354704</v>
+      </c>
+      <c r="W94" s="41" t="n">
+        <v>13.81884416310981</v>
+      </c>
+      <c r="X94" s="41" t="n">
+        <v>-0.5176839508974614</v>
+      </c>
+      <c r="Y94" s="41" t="n">
+        <v>-1.254462758512591</v>
+      </c>
+    </row>
+    <row r="95" ht="18.5" customHeight="1">
+      <c r="A95" s="56" t="n">
         <v>13</v>
       </c>
-      <c r="B67" s="37" t="n">
+      <c r="B95" s="37" t="n">
         <v>9.299592777273519</v>
       </c>
-      <c r="C67" s="37" t="n">
+      <c r="C95" s="37" t="n">
         <v>5.786159934187959</v>
       </c>
-      <c r="D67" s="37" t="n">
+      <c r="D95" s="37" t="n">
         <v>22.43116804942684</v>
       </c>
-      <c r="E67" s="37" t="n">
+      <c r="E95" s="37" t="n">
         <v>12.9516569707684</v>
       </c>
-      <c r="F67" s="37" t="n">
+      <c r="F95" s="37" t="n">
         <v>21.50223099093263</v>
       </c>
-      <c r="G67" s="37" t="n">
+      <c r="G95" s="37" t="n">
         <v>13.94854714691845</v>
       </c>
-      <c r="H67" s="37" t="n">
+      <c r="H95" s="37" t="n">
         <v>21.99197079914994</v>
       </c>
-      <c r="I67" s="37" t="n">
+      <c r="I95" s="37" t="n">
         <v>14.58115927506229</v>
       </c>
-      <c r="J67" s="37" t="n">
+      <c r="J95" s="37" t="n">
         <v>22.34755573117287</v>
       </c>
-      <c r="K67" s="37" t="n">
+      <c r="K95" s="37" t="n">
         <v>14.4250351982751</v>
       </c>
-    </row>
-    <row r="68" ht="18.5" customHeight="1">
-      <c r="A68" s="57" t="n">
+      <c r="L95" s="37" t="n">
+        <v>21.20656778610795</v>
+      </c>
+      <c r="M95" s="37" t="n">
+        <v>14.36877282314844</v>
+      </c>
+      <c r="N95" s="37" t="n">
+        <v>19.02167845942115</v>
+      </c>
+      <c r="O95" s="37" t="n">
+        <v>13.61986532073199</v>
+      </c>
+      <c r="P95" s="37" t="n">
+        <v>20.09664377296133</v>
+      </c>
+      <c r="Q95" s="37" t="n">
+        <v>14.30970600288065</v>
+      </c>
+      <c r="R95" s="37" t="n">
+        <v>18.78533221000992</v>
+      </c>
+      <c r="S95" s="37" t="n">
+        <v>13.41693055241567</v>
+      </c>
+      <c r="T95" s="37" t="n">
+        <v>20.5625543960503</v>
+      </c>
+      <c r="U95" s="37" t="n">
+        <v>13.53545115739081</v>
+      </c>
+      <c r="V95" s="37" t="n">
+        <v>20.46555025233066</v>
+      </c>
+      <c r="W95" s="37" t="n">
+        <v>13.9978000188436</v>
+      </c>
+      <c r="X95" s="37" t="n">
+        <v>3.442829987392189</v>
+      </c>
+      <c r="Y95" s="37" t="n">
+        <v>2.409810185195836</v>
+      </c>
+    </row>
+    <row r="96" ht="18.5" customHeight="1">
+      <c r="A96" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="B68" s="41" t="n">
+      <c r="B96" s="41" t="n">
         <v>9.917152719835924</v>
       </c>
-      <c r="C68" s="41" t="n">
+      <c r="C96" s="41" t="n">
         <v>6.243508232976811</v>
       </c>
-      <c r="D68" s="41" t="n">
+      <c r="D96" s="41" t="n">
         <v>23.23461799874261</v>
       </c>
-      <c r="E68" s="41" t="n">
+      <c r="E96" s="41" t="n">
         <v>13.15491574174829</v>
       </c>
-      <c r="F68" s="41" t="n">
+      <c r="F96" s="41" t="n">
         <v>21.96235281409825</v>
       </c>
-      <c r="G68" s="41" t="n">
+      <c r="G96" s="41" t="n">
         <v>13.9992324867488</v>
       </c>
-      <c r="H68" s="41" t="n">
+      <c r="H96" s="41" t="n">
         <v>22.11987722264312</v>
       </c>
-      <c r="I68" s="41" t="n">
+      <c r="I96" s="41" t="n">
         <v>14.48496053375388</v>
       </c>
-      <c r="J68" s="41" t="n">
+      <c r="J96" s="41" t="n">
         <v>22.7379543899728</v>
       </c>
-      <c r="K68" s="41" t="n">
+      <c r="K96" s="41" t="n">
         <v>14.69673743910437</v>
       </c>
-    </row>
-    <row r="69" ht="18.5" customHeight="1">
-      <c r="A69" s="56" t="n">
+      <c r="L96" s="41" t="n">
+        <v>21.44688401128137</v>
+      </c>
+      <c r="M96" s="41" t="n">
+        <v>14.45282271540129</v>
+      </c>
+      <c r="N96" s="41" t="n">
+        <v>19.31043546719657</v>
+      </c>
+      <c r="O96" s="41" t="n">
+        <v>13.54232422609503</v>
+      </c>
+      <c r="P96" s="41" t="n">
+        <v>20.12374462274371</v>
+      </c>
+      <c r="Q96" s="41" t="n">
+        <v>14.13987211765238</v>
+      </c>
+      <c r="R96" s="41" t="n">
+        <v>18.32751208011629</v>
+      </c>
+      <c r="S96" s="41" t="n">
+        <v>12.93977888431595</v>
+      </c>
+      <c r="T96" s="41" t="n">
+        <v>20.89571249638758</v>
+      </c>
+      <c r="U96" s="41" t="n">
+        <v>13.15143042163521</v>
+      </c>
+      <c r="V96" s="41" t="n">
+        <v>21.03682112636468</v>
+      </c>
+      <c r="W96" s="41" t="n">
+        <v>13.73789423055577</v>
+      </c>
+      <c r="X96" s="41" t="n">
+        <v>-1.445545489687058</v>
+      </c>
+      <c r="Y96" s="41" t="n">
+        <v>-2.096699960747216</v>
+      </c>
+    </row>
+    <row r="97" ht="18.5" customHeight="1">
+      <c r="A97" s="56" t="n">
         <v>15</v>
       </c>
-      <c r="B69" s="37" t="n">
+      <c r="B97" s="37" t="n">
         <v>11.25480292767549</v>
       </c>
-      <c r="C69" s="37" t="n">
+      <c r="C97" s="37" t="n">
         <v>6.802314489511978</v>
       </c>
-      <c r="D69" s="37" t="n">
+      <c r="D97" s="37" t="n">
         <v>24.23475829775696</v>
       </c>
-      <c r="E69" s="37" t="n">
+      <c r="E97" s="37" t="n">
         <v>13.26812103720495</v>
       </c>
-      <c r="F69" s="37" t="n">
+      <c r="F97" s="37" t="n">
         <v>22.84927299751978</v>
       </c>
-      <c r="G69" s="37" t="n">
+      <c r="G97" s="37" t="n">
         <v>14.19798565924701</v>
       </c>
-      <c r="H69" s="37" t="n">
+      <c r="H97" s="37" t="n">
         <v>22.92843775163052</v>
       </c>
-      <c r="I69" s="37" t="n">
+      <c r="I97" s="37" t="n">
         <v>14.72291597712155</v>
       </c>
-      <c r="J69" s="37" t="n">
+      <c r="J97" s="37" t="n">
         <v>23.48266563481791</v>
       </c>
-      <c r="K69" s="37" t="n">
+      <c r="K97" s="37" t="n">
         <v>14.8262195134175</v>
       </c>
-    </row>
-    <row r="70" ht="18.5" customHeight="1">
-      <c r="A70" s="57" t="n">
+      <c r="L97" s="37" t="n">
+        <v>22.24931515617125</v>
+      </c>
+      <c r="M97" s="37" t="n">
+        <v>14.62029289428374</v>
+      </c>
+      <c r="N97" s="37" t="n">
+        <v>20.20384137564892</v>
+      </c>
+      <c r="O97" s="37" t="n">
+        <v>14.02759181747573</v>
+      </c>
+      <c r="P97" s="37" t="n">
+        <v>21.12119380883288</v>
+      </c>
+      <c r="Q97" s="37" t="n">
+        <v>14.48441502003758</v>
+      </c>
+      <c r="R97" s="37" t="n">
+        <v>19.41236863512567</v>
+      </c>
+      <c r="S97" s="37" t="n">
+        <v>13.38034740493099</v>
+      </c>
+      <c r="T97" s="37" t="n">
+        <v>21.7876659661451</v>
+      </c>
+      <c r="U97" s="37" t="n">
+        <v>13.65959780073431</v>
+      </c>
+      <c r="V97" s="37" t="n">
+        <v>22.00612924502133</v>
+      </c>
+      <c r="W97" s="37" t="n">
+        <v>14.16494085212461</v>
+      </c>
+      <c r="X97" s="37" t="n">
+        <v>0.2145221711667503</v>
+      </c>
+      <c r="Y97" s="37" t="n">
+        <v>-0.9671779431820696</v>
+      </c>
+    </row>
+    <row r="98" ht="18.5" customHeight="1">
+      <c r="A98" s="57" t="n">
         <v>16</v>
       </c>
-      <c r="B70" s="41" t="n">
+      <c r="B98" s="41" t="n">
         <v>11.19072426992578</v>
       </c>
-      <c r="C70" s="41" t="n">
+      <c r="C98" s="41" t="n">
         <v>6.401623112000483</v>
       </c>
-      <c r="D70" s="41" t="n">
+      <c r="D98" s="41" t="n">
         <v>23.91467671017735</v>
       </c>
-      <c r="E70" s="41" t="n">
+      <c r="E98" s="41" t="n">
         <v>13.02338381548205</v>
       </c>
-      <c r="F70" s="41" t="n">
+      <c r="F98" s="41" t="n">
         <v>22.39478438248079</v>
       </c>
-      <c r="G70" s="41" t="n">
+      <c r="G98" s="41" t="n">
         <v>13.87100182808214</v>
       </c>
-      <c r="H70" s="41" t="n">
+      <c r="H98" s="41" t="n">
         <v>23.3420854612061</v>
       </c>
-      <c r="I70" s="41" t="n">
+      <c r="I98" s="41" t="n">
         <v>14.63020364331324</v>
       </c>
-      <c r="J70" s="41" t="n">
+      <c r="J98" s="41" t="n">
         <v>23.61021202319192</v>
       </c>
-      <c r="K70" s="41" t="n">
+      <c r="K98" s="41" t="n">
         <v>14.58349644880576</v>
       </c>
-    </row>
-    <row r="71" ht="18.5" customHeight="1">
-      <c r="A71" s="56" t="n">
+      <c r="L98" s="41" t="n">
+        <v>22.31231857368667</v>
+      </c>
+      <c r="M98" s="41" t="n">
+        <v>14.6965140171027</v>
+      </c>
+      <c r="N98" s="41" t="n">
+        <v>20.35826304403574</v>
+      </c>
+      <c r="O98" s="41" t="n">
+        <v>14.03595028265588</v>
+      </c>
+      <c r="P98" s="41" t="n">
+        <v>21.28185612268534</v>
+      </c>
+      <c r="Q98" s="41" t="n">
+        <v>14.4499915809962</v>
+      </c>
+      <c r="R98" s="41" t="n">
+        <v>19.6712554084745</v>
+      </c>
+      <c r="S98" s="41" t="n">
+        <v>13.60548352921847</v>
+      </c>
+      <c r="T98" s="41" t="n">
+        <v>22.18838219390685</v>
+      </c>
+      <c r="U98" s="41" t="n">
+        <v>13.69397126063065</v>
+      </c>
+      <c r="V98" s="41" t="n">
+        <v>22.11564649690117</v>
+      </c>
+      <c r="W98" s="41" t="n">
+        <v>14.09394349598651</v>
+      </c>
+      <c r="X98" s="41" t="n">
+        <v>3.186726563575667</v>
+      </c>
+      <c r="Y98" s="41" t="n">
+        <v>1.514255895898485</v>
+      </c>
+    </row>
+    <row r="99" ht="18.5" customHeight="1">
+      <c r="A99" s="56" t="n">
         <v>17</v>
       </c>
-      <c r="B71" s="37" t="n">
+      <c r="B99" s="37" t="n">
         <v>11.25457327267474</v>
       </c>
-      <c r="C71" s="37" t="n">
+      <c r="C99" s="37" t="n">
         <v>6.728193975011785</v>
       </c>
-      <c r="D71" s="37" t="n">
+      <c r="D99" s="37" t="n">
         <v>24.12938761420358</v>
       </c>
-      <c r="E71" s="37" t="n">
+      <c r="E99" s="37" t="n">
         <v>12.88619329634609</v>
       </c>
-      <c r="F71" s="37" t="n">
+      <c r="F99" s="37" t="n">
         <v>22.61313426331391</v>
       </c>
-      <c r="G71" s="37" t="n">
+      <c r="G99" s="37" t="n">
         <v>13.70338028851792</v>
       </c>
-      <c r="H71" s="37" t="n">
+      <c r="H99" s="37" t="n">
         <v>24.1132701734974</v>
       </c>
-      <c r="I71" s="37" t="n">
+      <c r="I99" s="37" t="n">
         <v>14.87129293097586</v>
       </c>
-      <c r="J71" s="37" t="n">
+      <c r="J99" s="37" t="n">
         <v>24.08764216133807</v>
       </c>
-      <c r="K71" s="37" t="n">
+      <c r="K99" s="37" t="n">
         <v>14.58378216733576</v>
       </c>
-    </row>
-    <row r="72" ht="18.5" customHeight="1">
-      <c r="A72" s="57" t="n">
+      <c r="L99" s="37" t="n">
+        <v>23.12956236199983</v>
+      </c>
+      <c r="M99" s="37" t="n">
+        <v>14.85086056556607</v>
+      </c>
+      <c r="N99" s="37" t="n">
+        <v>20.89584088540323</v>
+      </c>
+      <c r="O99" s="37" t="n">
+        <v>14.25144541311956</v>
+      </c>
+      <c r="P99" s="37" t="n">
+        <v>21.9695518403825</v>
+      </c>
+      <c r="Q99" s="37" t="n">
+        <v>14.64011972474557</v>
+      </c>
+      <c r="R99" s="37" t="n">
+        <v>20.73290581831791</v>
+      </c>
+      <c r="S99" s="37" t="n">
+        <v>13.98577139571209</v>
+      </c>
+      <c r="T99" s="37" t="n">
+        <v>22.14806359050422</v>
+      </c>
+      <c r="U99" s="37" t="n">
+        <v>13.60361552989039</v>
+      </c>
+      <c r="V99" s="37" t="n">
+        <v>22.91600738287404</v>
+      </c>
+      <c r="W99" s="37" t="n">
+        <v>14.37282242652016</v>
+      </c>
+      <c r="X99" s="37" t="n">
+        <v>1.164439041497553</v>
+      </c>
+      <c r="Y99" s="37" t="n">
+        <v>0.06378750143666097</v>
+      </c>
+    </row>
+    <row r="100" ht="18.5" customHeight="1">
+      <c r="A100" s="57" t="n">
         <v>18</v>
       </c>
-      <c r="B72" s="41" t="n">
+      <c r="B100" s="41" t="n">
         <v>11.97346633303058</v>
       </c>
-      <c r="C72" s="41" t="n">
+      <c r="C100" s="41" t="n">
         <v>7.001509639255496</v>
       </c>
-      <c r="D72" s="41" t="n">
+      <c r="D100" s="41" t="n">
         <v>24.95270292985132</v>
       </c>
-      <c r="E72" s="41" t="n">
+      <c r="E100" s="41" t="n">
         <v>13.02562497708743</v>
       </c>
-      <c r="F72" s="41" t="n">
+      <c r="F100" s="41" t="n">
         <v>23.52171033385683</v>
       </c>
-      <c r="G72" s="41" t="n">
+      <c r="G100" s="41" t="n">
         <v>14.03293195328007</v>
       </c>
-      <c r="H72" s="41" t="n">
+      <c r="H100" s="41" t="n">
         <v>24.22367413206014</v>
       </c>
-      <c r="I72" s="41" t="n">
+      <c r="I100" s="41" t="n">
         <v>14.73651360908862</v>
       </c>
-      <c r="J72" s="41" t="n">
+      <c r="J100" s="41" t="n">
         <v>24.41996550409049</v>
       </c>
-      <c r="K72" s="41" t="n">
+      <c r="K100" s="41" t="n">
         <v>14.77306331845293</v>
       </c>
-    </row>
-    <row r="73" ht="18.5" customHeight="1">
-      <c r="A73" s="56" t="n">
+      <c r="L100" s="41" t="n">
+        <v>23.19657800213909</v>
+      </c>
+      <c r="M100" s="41" t="n">
+        <v>14.69636413051092</v>
+      </c>
+      <c r="N100" s="41" t="n">
+        <v>21.18742943728228</v>
+      </c>
+      <c r="O100" s="41" t="n">
+        <v>14.24391988124458</v>
+      </c>
+      <c r="P100" s="41" t="n">
+        <v>22.19505249540916</v>
+      </c>
+      <c r="Q100" s="41" t="n">
+        <v>14.61651510985641</v>
+      </c>
+      <c r="R100" s="41" t="n">
+        <v>20.19899260663374</v>
+      </c>
+      <c r="S100" s="41" t="n">
+        <v>13.55597522906791</v>
+      </c>
+      <c r="T100" s="41" t="n">
+        <v>22.1631145985899</v>
+      </c>
+      <c r="U100" s="41" t="n">
+        <v>13.63473989223646</v>
+      </c>
+      <c r="V100" s="41" t="n">
+        <v>23.02296450306143</v>
+      </c>
+      <c r="W100" s="41" t="n">
+        <v>14.38610425362307</v>
+      </c>
+      <c r="X100" s="41" t="n">
+        <v>0.1152176835719707</v>
+      </c>
+      <c r="Y100" s="41" t="n">
+        <v>-0.5359982169933762</v>
+      </c>
+    </row>
+    <row r="101" ht="18.5" customHeight="1">
+      <c r="A101" s="56" t="n">
         <v>19</v>
       </c>
-      <c r="B73" s="37" t="n">
+      <c r="B101" s="37" t="n">
         <v>11.85607646845184</v>
       </c>
-      <c r="C73" s="37" t="n">
+      <c r="C101" s="37" t="n">
         <v>6.849180231385547</v>
       </c>
-      <c r="D73" s="37" t="n">
+      <c r="D101" s="37" t="n">
         <v>24.93908833037429</v>
       </c>
-      <c r="E73" s="37" t="n">
+      <c r="E101" s="37" t="n">
         <v>13.19448899129274</v>
       </c>
-      <c r="F73" s="37" t="n">
+      <c r="F101" s="37" t="n">
         <v>23.29666001847398</v>
       </c>
-      <c r="G73" s="37" t="n">
+      <c r="G101" s="37" t="n">
         <v>13.99658167850152</v>
       </c>
-      <c r="H73" s="37" t="n">
+      <c r="H101" s="37" t="n">
         <v>23.95292461396173</v>
       </c>
-      <c r="I73" s="37" t="n">
+      <c r="I101" s="37" t="n">
         <v>14.77169903537636</v>
       </c>
-      <c r="J73" s="37" t="n">
+      <c r="J101" s="37" t="n">
         <v>24.2245660291792</v>
       </c>
-      <c r="K73" s="37" t="n">
+      <c r="K101" s="37" t="n">
         <v>14.71697048669216</v>
       </c>
-    </row>
-    <row r="74" ht="18.5" customHeight="1">
-      <c r="A74" s="57" t="n">
+      <c r="L101" s="37" t="n">
+        <v>22.883802398729</v>
+      </c>
+      <c r="M101" s="37" t="n">
+        <v>14.68582619853975</v>
+      </c>
+      <c r="N101" s="37" t="n">
+        <v>20.91760861042161</v>
+      </c>
+      <c r="O101" s="37" t="n">
+        <v>14.28529709525752</v>
+      </c>
+      <c r="P101" s="37" t="n">
+        <v>22.09753688605602</v>
+      </c>
+      <c r="Q101" s="37" t="n">
+        <v>14.57805566813571</v>
+      </c>
+      <c r="R101" s="37" t="n">
+        <v>20.16650404697691</v>
+      </c>
+      <c r="S101" s="37" t="n">
+        <v>13.61504579373341</v>
+      </c>
+      <c r="T101" s="37" t="n">
+        <v>22.35788307914904</v>
+      </c>
+      <c r="U101" s="37" t="n">
+        <v>13.82473528253288</v>
+      </c>
+      <c r="V101" s="37" t="n">
+        <v>23.03417147667185</v>
+      </c>
+      <c r="W101" s="37" t="n">
+        <v>14.5230454750158</v>
+      </c>
+      <c r="X101" s="37" t="n">
+        <v>2.649077556286063</v>
+      </c>
+      <c r="Y101" s="37" t="n">
+        <v>1.371305640656699</v>
+      </c>
+    </row>
+    <row r="102" ht="18.5" customHeight="1">
+      <c r="A102" s="57" t="n">
         <v>20</v>
       </c>
-      <c r="B74" s="41" t="n">
+      <c r="B102" s="41" t="n">
         <v>12.00633881121406</v>
       </c>
-      <c r="C74" s="41" t="n">
+      <c r="C102" s="41" t="n">
         <v>6.828583097040846</v>
       </c>
-      <c r="D74" s="41" t="n">
+      <c r="D102" s="41" t="n">
         <v>25.17345260353249</v>
       </c>
-      <c r="E74" s="41" t="n">
+      <c r="E102" s="41" t="n">
         <v>13.37635003135219</v>
       </c>
-      <c r="F74" s="41" t="n">
+      <c r="F102" s="41" t="n">
         <v>23.66022120977462</v>
       </c>
-      <c r="G74" s="41" t="n">
+      <c r="G102" s="41" t="n">
         <v>14.3010184878057</v>
       </c>
-      <c r="H74" s="41" t="n">
+      <c r="H102" s="41" t="n">
         <v>24.17808655746551</v>
       </c>
-      <c r="I74" s="41" t="n">
+      <c r="I102" s="41" t="n">
         <v>14.96028532538482</v>
       </c>
-      <c r="J74" s="41" t="n">
+      <c r="J102" s="41" t="n">
         <v>24.50974142979358</v>
       </c>
-      <c r="K74" s="41" t="n">
+      <c r="K102" s="41" t="n">
         <v>14.97365913393347</v>
+      </c>
+      <c r="L102" s="41" t="n">
+        <v>23.08604968955818</v>
+      </c>
+      <c r="M102" s="41" t="n">
+        <v>14.86219420698205</v>
+      </c>
+      <c r="N102" s="41" t="n">
+        <v>21.00177536491885</v>
+      </c>
+      <c r="O102" s="41" t="n">
+        <v>14.39484412181733</v>
+      </c>
+      <c r="P102" s="41" t="n">
+        <v>22.14820816691532</v>
+      </c>
+      <c r="Q102" s="41" t="n">
+        <v>14.72664831686643</v>
+      </c>
+      <c r="R102" s="41" t="n">
+        <v>20.42072947846276</v>
+      </c>
+      <c r="S102" s="41" t="n">
+        <v>13.83451629399157</v>
+      </c>
+      <c r="T102" s="41" t="n">
+        <v>22.05969672189216</v>
+      </c>
+      <c r="U102" s="41" t="n">
+        <v>13.60311970521846</v>
+      </c>
+      <c r="V102" s="41" t="n">
+        <v>22.71705389740357</v>
+      </c>
+      <c r="W102" s="41" t="n">
+        <v>14.25407969386831</v>
+      </c>
+      <c r="X102" s="41" t="n">
+        <v>3.001832752684395</v>
+      </c>
+      <c r="Y102" s="41" t="n">
+        <v>1.769338035541456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>